<commit_message>
Add extract_scores.py and seed Match Results / Team Stats sheets
- extract_scores.py fetches WC2026 match data from football-data.org (free tier)
  and applies the full scoring rules to each participant's picks
- --mock flag runs with bundled sample data covering group stage, AET/pens,
  and future scheduled matches so the pipeline can be tested without an API key
- Writes three sheets to WC2026_Pool.xlsx:
    Match Results  – all matches with scores, stage, group, duration, status
    Team Stats     – per-team points, goals, and bonus breakdown
    Scoring        – TOTAL PTS column now populated from computed standings
- Run: python extract_scores.py --mock
        python extract_scores.py --api-key YOUR_KEY  (or set FOOTBALL_DATA_API_KEY)

https://claude.ai/code/session_01VFqgqUhDsMbhjQyNveqHky
</commit_message>
<xml_diff>
--- a/WC2026_Pool.xlsx
+++ b/WC2026_Pool.xlsx
@@ -11,6 +11,8 @@
     <sheet name="Scoring Rules" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Entrants" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Scoring" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Match Results" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Team Stats" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -413,7 +415,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -583,6 +585,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2818,7 +2823,9 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="N3" s="58" t="n"/>
+      <c r="N3" s="58" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="4" ht="18" customHeight="1" s="28">
       <c r="A4" s="59" t="inlineStr">
@@ -2886,7 +2893,9 @@
           <t>Iraq</t>
         </is>
       </c>
-      <c r="N4" s="58" t="n"/>
+      <c r="N4" s="58" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1" s="28">
       <c r="A5" s="56" t="inlineStr">
@@ -2954,7 +2963,9 @@
           <t>DR Congo</t>
         </is>
       </c>
-      <c r="N5" s="58" t="n"/>
+      <c r="N5" s="58" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="6" ht="18" customHeight="1" s="28">
       <c r="A6" s="59" t="inlineStr">
@@ -3022,7 +3033,9 @@
           <t>Iraq</t>
         </is>
       </c>
-      <c r="N6" s="58" t="n"/>
+      <c r="N6" s="58" t="n">
+        <v>38</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3030,4 +3043,1151 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="28" min="1" max="1"/>
+    <col width="16" customWidth="1" style="28" min="2" max="2"/>
+    <col width="10" customWidth="1" style="28" min="3" max="3"/>
+    <col width="20" customWidth="1" style="28" min="4" max="4"/>
+    <col width="10" customWidth="1" style="28" min="5" max="5"/>
+    <col width="20" customWidth="1" style="28" min="6" max="6"/>
+    <col width="14" customWidth="1" style="28" min="7" max="7"/>
+    <col width="20" customWidth="1" style="28" min="8" max="8"/>
+    <col width="12" customWidth="1" style="28" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="61" t="inlineStr">
+        <is>
+          <t>Date (UTC)</t>
+        </is>
+      </c>
+      <c r="B1" s="61" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C1" s="61" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D1" s="61" t="inlineStr">
+        <is>
+          <t>Home Team</t>
+        </is>
+      </c>
+      <c r="E1" s="61" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="F1" s="61" t="inlineStr">
+        <is>
+          <t>Away Team</t>
+        </is>
+      </c>
+      <c r="G1" s="61" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="H1" s="61" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="I1" s="61" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="57" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B2" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_STAGE</t>
+        </is>
+      </c>
+      <c r="C2" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_A</t>
+        </is>
+      </c>
+      <c r="D2" s="57" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E2" s="57" t="inlineStr">
+        <is>
+          <t>2 – 1</t>
+        </is>
+      </c>
+      <c r="F2" s="57" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="G2" s="57" t="inlineStr">
+        <is>
+          <t>HOME_TEAM</t>
+        </is>
+      </c>
+      <c r="H2" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I2" s="57" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B3" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_STAGE</t>
+        </is>
+      </c>
+      <c r="C3" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_A</t>
+        </is>
+      </c>
+      <c r="D3" s="60" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="E3" s="60" t="inlineStr">
+        <is>
+          <t>0 – 0</t>
+        </is>
+      </c>
+      <c r="F3" s="60" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="G3" s="60" t="inlineStr">
+        <is>
+          <t>DRAW</t>
+        </is>
+      </c>
+      <c r="H3" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I3" s="60" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="57" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B4" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_STAGE</t>
+        </is>
+      </c>
+      <c r="C4" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_B</t>
+        </is>
+      </c>
+      <c r="D4" s="57" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="E4" s="57" t="inlineStr">
+        <is>
+          <t>2 – 0</t>
+        </is>
+      </c>
+      <c r="F4" s="57" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herz.</t>
+        </is>
+      </c>
+      <c r="G4" s="57" t="inlineStr">
+        <is>
+          <t>HOME_TEAM</t>
+        </is>
+      </c>
+      <c r="H4" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I4" s="57" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B5" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_STAGE</t>
+        </is>
+      </c>
+      <c r="C5" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_B</t>
+        </is>
+      </c>
+      <c r="D5" s="60" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E5" s="60" t="inlineStr">
+        <is>
+          <t>3 – 1</t>
+        </is>
+      </c>
+      <c r="F5" s="60" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="G5" s="60" t="inlineStr">
+        <is>
+          <t>HOME_TEAM</t>
+        </is>
+      </c>
+      <c r="H5" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I5" s="60" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="57" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B6" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_STAGE</t>
+        </is>
+      </c>
+      <c r="C6" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_A</t>
+        </is>
+      </c>
+      <c r="D6" s="57" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E6" s="57" t="inlineStr">
+        <is>
+          <t>3 – 0</t>
+        </is>
+      </c>
+      <c r="F6" s="57" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G6" s="57" t="inlineStr">
+        <is>
+          <t>HOME_TEAM</t>
+        </is>
+      </c>
+      <c r="H6" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I6" s="57" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B7" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_STAGE</t>
+        </is>
+      </c>
+      <c r="C7" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_A</t>
+        </is>
+      </c>
+      <c r="D7" s="60" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="E7" s="60" t="inlineStr">
+        <is>
+          <t>1 – 2</t>
+        </is>
+      </c>
+      <c r="F7" s="60" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="G7" s="60" t="inlineStr">
+        <is>
+          <t>AWAY_TEAM</t>
+        </is>
+      </c>
+      <c r="H7" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I7" s="60" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="57" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B8" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_STAGE</t>
+        </is>
+      </c>
+      <c r="C8" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_B</t>
+        </is>
+      </c>
+      <c r="D8" s="57" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="E8" s="57" t="inlineStr">
+        <is>
+          <t>4 – 0</t>
+        </is>
+      </c>
+      <c r="F8" s="57" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="G8" s="57" t="inlineStr">
+        <is>
+          <t>HOME_TEAM</t>
+        </is>
+      </c>
+      <c r="H8" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I8" s="57" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B9" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_STAGE</t>
+        </is>
+      </c>
+      <c r="C9" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_B</t>
+        </is>
+      </c>
+      <c r="D9" s="60" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E9" s="60" t="inlineStr">
+        <is>
+          <t>2 – 2</t>
+        </is>
+      </c>
+      <c r="F9" s="60" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herz.</t>
+        </is>
+      </c>
+      <c r="G9" s="60" t="inlineStr">
+        <is>
+          <t>DRAW</t>
+        </is>
+      </c>
+      <c r="H9" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I9" s="60" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="57" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B10" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_STAGE</t>
+        </is>
+      </c>
+      <c r="C10" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_A</t>
+        </is>
+      </c>
+      <c r="D10" s="57" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E10" s="57" t="inlineStr">
+        <is>
+          <t>1 – 0</t>
+        </is>
+      </c>
+      <c r="F10" s="57" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="G10" s="57" t="inlineStr">
+        <is>
+          <t>HOME_TEAM</t>
+        </is>
+      </c>
+      <c r="H10" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I10" s="57" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B11" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_STAGE</t>
+        </is>
+      </c>
+      <c r="C11" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_A</t>
+        </is>
+      </c>
+      <c r="D11" s="60" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="E11" s="60" t="inlineStr">
+        <is>
+          <t>1 – 2</t>
+        </is>
+      </c>
+      <c r="F11" s="60" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="G11" s="60" t="inlineStr">
+        <is>
+          <t>AWAY_TEAM</t>
+        </is>
+      </c>
+      <c r="H11" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I11" s="60" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="57" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B12" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_STAGE</t>
+        </is>
+      </c>
+      <c r="C12" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_B</t>
+        </is>
+      </c>
+      <c r="D12" s="57" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="E12" s="57" t="inlineStr">
+        <is>
+          <t>1 – 2</t>
+        </is>
+      </c>
+      <c r="F12" s="57" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="G12" s="57" t="inlineStr">
+        <is>
+          <t>AWAY_TEAM</t>
+        </is>
+      </c>
+      <c r="H12" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I12" s="57" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="60" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B13" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_STAGE</t>
+        </is>
+      </c>
+      <c r="C13" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_B</t>
+        </is>
+      </c>
+      <c r="D13" s="60" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herz.</t>
+        </is>
+      </c>
+      <c r="E13" s="60" t="inlineStr">
+        <is>
+          <t>2 – 1</t>
+        </is>
+      </c>
+      <c r="F13" s="60" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="G13" s="60" t="inlineStr">
+        <is>
+          <t>HOME_TEAM</t>
+        </is>
+      </c>
+      <c r="H13" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I13" s="60" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="57" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B14" s="57" t="inlineStr">
+        <is>
+          <t>LAST_16</t>
+        </is>
+      </c>
+      <c r="C14" s="57" t="inlineStr"/>
+      <c r="D14" s="57" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E14" s="57" t="inlineStr">
+        <is>
+          <t>1 – 1</t>
+        </is>
+      </c>
+      <c r="F14" s="57" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="G14" s="57" t="inlineStr">
+        <is>
+          <t>HOME_TEAM</t>
+        </is>
+      </c>
+      <c r="H14" s="57" t="inlineStr">
+        <is>
+          <t>PENALTY_SHOOTOUT</t>
+        </is>
+      </c>
+      <c r="I14" s="57" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="60" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B15" s="60" t="inlineStr">
+        <is>
+          <t>LAST_16</t>
+        </is>
+      </c>
+      <c r="C15" s="60" t="inlineStr"/>
+      <c r="D15" s="60" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="E15" s="60" t="inlineStr">
+        <is>
+          <t>2 – 0</t>
+        </is>
+      </c>
+      <c r="F15" s="60" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="G15" s="60" t="inlineStr">
+        <is>
+          <t>HOME_TEAM</t>
+        </is>
+      </c>
+      <c r="H15" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I15" s="60" t="inlineStr">
+        <is>
+          <t>FINISHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="57" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B16" s="57" t="inlineStr">
+        <is>
+          <t>LAST_16</t>
+        </is>
+      </c>
+      <c r="C16" s="57" t="inlineStr"/>
+      <c r="D16" s="57" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E16" s="57" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F16" s="57" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="G16" s="57" t="inlineStr"/>
+      <c r="H16" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="I16" s="57" t="inlineStr">
+        <is>
+          <t>SCHEDULED</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" style="28" min="1" max="1"/>
+    <col width="10" customWidth="1" style="28" min="2" max="2"/>
+    <col width="16" customWidth="1" style="28" min="3" max="3"/>
+    <col width="18" customWidth="1" style="28" min="4" max="4"/>
+    <col width="20" customWidth="1" style="28" min="5" max="5"/>
+    <col width="10" customWidth="1" style="28" min="6" max="6"/>
+    <col width="10" customWidth="1" style="28" min="7" max="7"/>
+    <col width="10" customWidth="1" style="28" min="8" max="8"/>
+    <col width="45" customWidth="1" style="28" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="61" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="B1" s="61" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C1" s="61" t="inlineStr">
+        <is>
+          <t>Matches Played</t>
+        </is>
+      </c>
+      <c r="D1" s="61" t="inlineStr">
+        <is>
+          <t>Gp Goals Scored</t>
+        </is>
+      </c>
+      <c r="E1" s="61" t="inlineStr">
+        <is>
+          <t>Gp Goals Conceded</t>
+        </is>
+      </c>
+      <c r="F1" s="61" t="inlineStr">
+        <is>
+          <t>Match Pts</t>
+        </is>
+      </c>
+      <c r="G1" s="61" t="inlineStr">
+        <is>
+          <t>Bonus Pts</t>
+        </is>
+      </c>
+      <c r="H1" s="61" t="inlineStr">
+        <is>
+          <t>Total Pts</t>
+        </is>
+      </c>
+      <c r="I1" s="61" t="inlineStr">
+        <is>
+          <t>Bonus Breakdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="57" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="B2" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_A</t>
+        </is>
+      </c>
+      <c r="C2" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" s="57" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="57" t="n">
+        <v>9</v>
+      </c>
+      <c r="G2" s="57" t="n">
+        <v>12</v>
+      </c>
+      <c r="H2" s="57" t="n">
+        <v>21</v>
+      </c>
+      <c r="I2" s="57" t="inlineStr">
+        <is>
+          <t>group_winner(+3), top_scorer_group(+3), best_defense_group(+3), best_defense_tournament(+3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="60" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B3" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_B</t>
+        </is>
+      </c>
+      <c r="C3" s="60" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" s="60" t="n">
+        <v>7</v>
+      </c>
+      <c r="E3" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="60" t="n">
+        <v>7</v>
+      </c>
+      <c r="G3" s="60" t="n">
+        <v>12</v>
+      </c>
+      <c r="H3" s="60" t="n">
+        <v>19</v>
+      </c>
+      <c r="I3" s="60" t="inlineStr">
+        <is>
+          <t>group_winner(+3), top_scorer_group(+3), top_scorer_tournament(+3), best_defense_group(+3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="57" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B4" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_B</t>
+        </is>
+      </c>
+      <c r="C4" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" s="57" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" s="57" t="n">
+        <v>7</v>
+      </c>
+      <c r="G4" s="57" t="n">
+        <v>9</v>
+      </c>
+      <c r="H4" s="57" t="n">
+        <v>16</v>
+      </c>
+      <c r="I4" s="57" t="inlineStr">
+        <is>
+          <t>group_winner(+3), top_scorer_group(+3), top_scorer_tournament(+3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="60" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="B5" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_A</t>
+        </is>
+      </c>
+      <c r="C5" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="60" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="60" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" s="60" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="57" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herz.</t>
+        </is>
+      </c>
+      <c r="B6" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_B</t>
+        </is>
+      </c>
+      <c r="C6" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="57" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" s="57" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="60" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="B7" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_A</t>
+        </is>
+      </c>
+      <c r="C7" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="60" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="60" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="60" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="57" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B8" s="57" t="inlineStr"/>
+      <c r="C8" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" s="57" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="60" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="B9" s="60" t="inlineStr"/>
+      <c r="C9" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" s="60" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="57" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="B10" s="57" t="inlineStr">
+        <is>
+          <t>GROUP_A</t>
+        </is>
+      </c>
+      <c r="C10" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="57" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="57" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="60" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="B11" s="60" t="inlineStr">
+        <is>
+          <t>GROUP_B</t>
+        </is>
+      </c>
+      <c r="C11" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="60" t="n">
+        <v>9</v>
+      </c>
+      <c r="F11" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="60" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add statistics.py and Statistics tab to master workbook
- statistics.py tallies how many participants picked each team, grouped by
  tier and sorted by descending pick count within each tier
- Statistics tab in WC2026_Pool.xlsx shows: Tier, Team, WC Group, # Picked,
  % Picked, and which participants chose that team
- Tier section headers and pastel row fills use each tier's colour
- Console output includes an ASCII bar chart for quick review
- 28 of 48 teams were picked; Spain/Norway/Switzerland/Sweden/Canada each
  attracted 3 of 4 participants

https://claude.ai/code/session_01VFqgqUhDsMbhjQyNveqHky
</commit_message>
<xml_diff>
--- a/WC2026_Pool.xlsx
+++ b/WC2026_Pool.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Scoring" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Match Results" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Team Stats" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Statistics" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="28">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -197,8 +198,18 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="25">
+  <fills count="31">
     <fill>
       <patternFill/>
     </fill>
@@ -320,6 +331,36 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3D1D1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9E4D2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBE0D7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5DBE2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E5D9ED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E1E1E1"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="8">
     <border>
@@ -415,7 +456,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -589,6 +630,81 @@
     </xf>
     <xf numFmtId="0" fontId="26" fillId="15" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4190,4 +4306,1556 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" style="28" min="1" max="1"/>
+    <col width="20" customWidth="1" style="28" min="2" max="2"/>
+    <col width="12" customWidth="1" style="28" min="3" max="3"/>
+    <col width="10" customWidth="1" style="28" min="4" max="4"/>
+    <col width="10" customWidth="1" style="28" min="5" max="5"/>
+    <col width="50" customWidth="1" style="28" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" s="28">
+      <c r="A1" s="62" t="inlineStr">
+        <is>
+          <t>2026 FIFA World Cup Pool – Team Pick Statistics  (4 participants)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1" s="28">
+      <c r="A2" s="61" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B2" s="61" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="C2" s="61" t="inlineStr">
+        <is>
+          <t>WC Group</t>
+        </is>
+      </c>
+      <c r="D2" s="61" t="inlineStr">
+        <is>
+          <t># Picked</t>
+        </is>
+      </c>
+      <c r="E2" s="61" t="inlineStr">
+        <is>
+          <t>% Picked</t>
+        </is>
+      </c>
+      <c r="F2" s="61" t="inlineStr">
+        <is>
+          <t>Picked By</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1" s="28">
+      <c r="A3" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tier 1 – Elite Favorites</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1" s="28">
+      <c r="A4" s="64" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="B4" s="64" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C4" s="64" t="inlineStr">
+        <is>
+          <t>Group H</t>
+        </is>
+      </c>
+      <c r="D4" s="65" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="64" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="F4" s="66" t="inlineStr">
+        <is>
+          <t>Ken Larade, Ryan Lowe, Lucie Kendell</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1" s="28">
+      <c r="A5" s="64" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="B5" s="64" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C5" s="64" t="inlineStr">
+        <is>
+          <t>Group I</t>
+        </is>
+      </c>
+      <c r="D5" s="65" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="64" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="F5" s="66" t="inlineStr">
+        <is>
+          <t>Ken Larade, Peter Miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1" s="28">
+      <c r="A6" s="64" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="B6" s="64" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C6" s="64" t="inlineStr">
+        <is>
+          <t>Group J</t>
+        </is>
+      </c>
+      <c r="D6" s="65" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="64" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F6" s="66" t="inlineStr">
+        <is>
+          <t>Ryan Lowe</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1" s="28">
+      <c r="A7" s="64" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="B7" s="64" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C7" s="64" t="inlineStr">
+        <is>
+          <t>Group L</t>
+        </is>
+      </c>
+      <c r="D7" s="65" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="64" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F7" s="66" t="inlineStr">
+        <is>
+          <t>Lucie Kendell</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1" s="28">
+      <c r="A8" s="64" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="B8" s="64" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C8" s="64" t="inlineStr">
+        <is>
+          <t>Group K</t>
+        </is>
+      </c>
+      <c r="D8" s="65" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="64" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F8" s="66" t="inlineStr">
+        <is>
+          <t>Peter Miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1" s="28">
+      <c r="A9" s="64" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="B9" s="64" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="C9" s="64" t="inlineStr">
+        <is>
+          <t>Group C</t>
+        </is>
+      </c>
+      <c r="D9" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="64" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F9" s="66" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1" s="28">
+      <c r="A10" s="64" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="B10" s="64" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C10" s="64" t="inlineStr">
+        <is>
+          <t>Group E</t>
+        </is>
+      </c>
+      <c r="D10" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="64" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F10" s="66" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1" s="28">
+      <c r="A11" s="64" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="B11" s="64" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="C11" s="64" t="inlineStr">
+        <is>
+          <t>Group F</t>
+        </is>
+      </c>
+      <c r="D11" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="64" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F11" s="66" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="28">
+      <c r="A12" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tier 2 – Contenders</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1" s="28">
+      <c r="A13" s="68" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="B13" s="68" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="C13" s="68" t="inlineStr">
+        <is>
+          <t>Group G</t>
+        </is>
+      </c>
+      <c r="D13" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="68" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="F13" s="70" t="inlineStr">
+        <is>
+          <t>Ken Larade, Lucie Kendell</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1" s="28">
+      <c r="A14" s="68" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="B14" s="68" t="inlineStr">
+        <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="C14" s="68" t="inlineStr">
+        <is>
+          <t>Group L</t>
+        </is>
+      </c>
+      <c r="D14" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="68" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="F14" s="70" t="inlineStr">
+        <is>
+          <t>Ken Larade, Ryan Lowe</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1" s="28">
+      <c r="A15" s="68" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="B15" s="68" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="C15" s="68" t="inlineStr">
+        <is>
+          <t>Group C</t>
+        </is>
+      </c>
+      <c r="D15" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="68" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="F15" s="70" t="inlineStr">
+        <is>
+          <t>Ryan Lowe, Peter Miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1" s="28">
+      <c r="A16" s="68" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="B16" s="68" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C16" s="68" t="inlineStr">
+        <is>
+          <t>Group F</t>
+        </is>
+      </c>
+      <c r="D16" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="68" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F16" s="70" t="inlineStr">
+        <is>
+          <t>Peter Miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1" s="28">
+      <c r="A17" s="68" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="B17" s="68" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="C17" s="68" t="inlineStr">
+        <is>
+          <t>Group K</t>
+        </is>
+      </c>
+      <c r="D17" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="68" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F17" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1" s="28">
+      <c r="A18" s="68" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="B18" s="68" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C18" s="68" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="D18" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="68" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F18" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1" s="28">
+      <c r="A19" s="68" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="B19" s="68" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C19" s="68" t="inlineStr">
+        <is>
+          <t>Group D</t>
+        </is>
+      </c>
+      <c r="D19" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="68" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F19" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1" s="28">
+      <c r="A20" s="68" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="B20" s="68" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="C20" s="68" t="inlineStr">
+        <is>
+          <t>Group H</t>
+        </is>
+      </c>
+      <c r="D20" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="68" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F20" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="28">
+      <c r="A21" s="71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tier 3 – Dark Horses</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1" s="28">
+      <c r="A22" s="72" t="inlineStr">
+        <is>
+          <t>Tier 3</t>
+        </is>
+      </c>
+      <c r="B22" s="72" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="C22" s="72" t="inlineStr">
+        <is>
+          <t>Group I</t>
+        </is>
+      </c>
+      <c r="D22" s="73" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="72" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="F22" s="74" t="inlineStr">
+        <is>
+          <t>Ken Larade, Lucie Kendell, Peter Miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1" s="28">
+      <c r="A23" s="72" t="inlineStr">
+        <is>
+          <t>Tier 3</t>
+        </is>
+      </c>
+      <c r="B23" s="72" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C23" s="72" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="D23" s="73" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" s="72" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="F23" s="74" t="inlineStr">
+        <is>
+          <t>Ryan Lowe, Lucie Kendell, Peter Miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1" s="28">
+      <c r="A24" s="72" t="inlineStr">
+        <is>
+          <t>Tier 3</t>
+        </is>
+      </c>
+      <c r="B24" s="72" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="C24" s="72" t="inlineStr">
+        <is>
+          <t>Group E</t>
+        </is>
+      </c>
+      <c r="D24" s="73" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="72" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F24" s="74" t="inlineStr">
+        <is>
+          <t>Ryan Lowe</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1" s="28">
+      <c r="A25" s="72" t="inlineStr">
+        <is>
+          <t>Tier 3</t>
+        </is>
+      </c>
+      <c r="B25" s="72" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="C25" s="72" t="inlineStr">
+        <is>
+          <t>Group D</t>
+        </is>
+      </c>
+      <c r="D25" s="73" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="72" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F25" s="74" t="inlineStr">
+        <is>
+          <t>Ken Larade</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1" s="28">
+      <c r="A26" s="72" t="inlineStr">
+        <is>
+          <t>Tier 3</t>
+        </is>
+      </c>
+      <c r="B26" s="72" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="C26" s="72" t="inlineStr">
+        <is>
+          <t>Group J</t>
+        </is>
+      </c>
+      <c r="D26" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="72" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F26" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1" s="28">
+      <c r="A27" s="72" t="inlineStr">
+        <is>
+          <t>Tier 3</t>
+        </is>
+      </c>
+      <c r="B27" s="72" t="inlineStr">
+        <is>
+          <t>Ivory Coast</t>
+        </is>
+      </c>
+      <c r="C27" s="72" t="inlineStr">
+        <is>
+          <t>Group E</t>
+        </is>
+      </c>
+      <c r="D27" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="72" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F27" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1" s="28">
+      <c r="A28" s="72" t="inlineStr">
+        <is>
+          <t>Tier 3</t>
+        </is>
+      </c>
+      <c r="B28" s="72" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="C28" s="72" t="inlineStr">
+        <is>
+          <t>Group I</t>
+        </is>
+      </c>
+      <c r="D28" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="72" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F28" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1" s="28">
+      <c r="A29" s="72" t="inlineStr">
+        <is>
+          <t>Tier 3</t>
+        </is>
+      </c>
+      <c r="B29" s="72" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="C29" s="72" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="D29" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="72" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F29" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1" s="28">
+      <c r="A30" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tier 4 – Long Shots</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1" s="28">
+      <c r="A31" s="76" t="inlineStr">
+        <is>
+          <t>Tier 4</t>
+        </is>
+      </c>
+      <c r="B31" s="76" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C31" s="76" t="inlineStr">
+        <is>
+          <t>Group F</t>
+        </is>
+      </c>
+      <c r="D31" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" s="76" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="F31" s="78" t="inlineStr">
+        <is>
+          <t>Ryan Lowe, Lucie Kendell, Peter Miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1" s="28">
+      <c r="A32" s="76" t="inlineStr">
+        <is>
+          <t>Tier 4</t>
+        </is>
+      </c>
+      <c r="B32" s="76" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="C32" s="76" t="inlineStr">
+        <is>
+          <t>Group G</t>
+        </is>
+      </c>
+      <c r="D32" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="76" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="F32" s="78" t="inlineStr">
+        <is>
+          <t>Lucie Kendell, Peter Miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1" s="28">
+      <c r="A33" s="76" t="inlineStr">
+        <is>
+          <t>Tier 4</t>
+        </is>
+      </c>
+      <c r="B33" s="76" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="C33" s="76" t="inlineStr">
+        <is>
+          <t>Group J</t>
+        </is>
+      </c>
+      <c r="D33" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="76" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F33" s="78" t="inlineStr">
+        <is>
+          <t>Ken Larade</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="16" customHeight="1" s="28">
+      <c r="A34" s="76" t="inlineStr">
+        <is>
+          <t>Tier 4</t>
+        </is>
+      </c>
+      <c r="B34" s="76" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="C34" s="76" t="inlineStr">
+        <is>
+          <t>Group D</t>
+        </is>
+      </c>
+      <c r="D34" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="76" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F34" s="78" t="inlineStr">
+        <is>
+          <t>Ryan Lowe</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1" s="28">
+      <c r="A35" s="76" t="inlineStr">
+        <is>
+          <t>Tier 4</t>
+        </is>
+      </c>
+      <c r="B35" s="76" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C35" s="76" t="inlineStr">
+        <is>
+          <t>Group L</t>
+        </is>
+      </c>
+      <c r="D35" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="76" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F35" s="78" t="inlineStr">
+        <is>
+          <t>Ken Larade</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="16" customHeight="1" s="28">
+      <c r="A36" s="76" t="inlineStr">
+        <is>
+          <t>Tier 4</t>
+        </is>
+      </c>
+      <c r="B36" s="76" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="C36" s="76" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="D36" s="76" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="76" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F36" s="78" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="16" customHeight="1" s="28">
+      <c r="A37" s="76" t="inlineStr">
+        <is>
+          <t>Tier 4</t>
+        </is>
+      </c>
+      <c r="B37" s="76" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="C37" s="76" t="inlineStr">
+        <is>
+          <t>Group G</t>
+        </is>
+      </c>
+      <c r="D37" s="76" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="76" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F37" s="78" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="16" customHeight="1" s="28">
+      <c r="A38" s="76" t="inlineStr">
+        <is>
+          <t>Tier 4</t>
+        </is>
+      </c>
+      <c r="B38" s="76" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="C38" s="76" t="inlineStr">
+        <is>
+          <t>Group D</t>
+        </is>
+      </c>
+      <c r="D38" s="76" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="76" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F38" s="78" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1" s="28">
+      <c r="A39" s="79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tier 5 – Underdogs</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16" customHeight="1" s="28">
+      <c r="A40" s="80" t="inlineStr">
+        <is>
+          <t>Tier 5</t>
+        </is>
+      </c>
+      <c r="B40" s="80" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C40" s="80" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="D40" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" s="80" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="F40" s="82" t="inlineStr">
+        <is>
+          <t>Ken Larade, Lucie Kendell, Peter Miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="16" customHeight="1" s="28">
+      <c r="A41" s="80" t="inlineStr">
+        <is>
+          <t>Tier 5</t>
+        </is>
+      </c>
+      <c r="B41" s="80" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="C41" s="80" t="inlineStr">
+        <is>
+          <t>Group C</t>
+        </is>
+      </c>
+      <c r="D41" s="81" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="80" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="F41" s="82" t="inlineStr">
+        <is>
+          <t>Ken Larade, Peter Miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="16" customHeight="1" s="28">
+      <c r="A42" s="80" t="inlineStr">
+        <is>
+          <t>Tier 5</t>
+        </is>
+      </c>
+      <c r="B42" s="80" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C42" s="80" t="inlineStr">
+        <is>
+          <t>Group G</t>
+        </is>
+      </c>
+      <c r="D42" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="80" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F42" s="82" t="inlineStr">
+        <is>
+          <t>Ryan Lowe</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="16" customHeight="1" s="28">
+      <c r="A43" s="80" t="inlineStr">
+        <is>
+          <t>Tier 5</t>
+        </is>
+      </c>
+      <c r="B43" s="80" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="C43" s="80" t="inlineStr">
+        <is>
+          <t>Group H</t>
+        </is>
+      </c>
+      <c r="D43" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="80" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F43" s="82" t="inlineStr">
+        <is>
+          <t>Lucie Kendell</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="16" customHeight="1" s="28">
+      <c r="A44" s="80" t="inlineStr">
+        <is>
+          <t>Tier 5</t>
+        </is>
+      </c>
+      <c r="B44" s="80" t="inlineStr">
+        <is>
+          <t>Uzbekistan</t>
+        </is>
+      </c>
+      <c r="C44" s="80" t="inlineStr">
+        <is>
+          <t>Group K</t>
+        </is>
+      </c>
+      <c r="D44" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="80" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F44" s="82" t="inlineStr">
+        <is>
+          <t>Ryan Lowe</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="16" customHeight="1" s="28">
+      <c r="A45" s="80" t="inlineStr">
+        <is>
+          <t>Tier 5</t>
+        </is>
+      </c>
+      <c r="B45" s="80" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herz.</t>
+        </is>
+      </c>
+      <c r="C45" s="80" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="D45" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="80" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F45" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="16" customHeight="1" s="28">
+      <c r="A46" s="80" t="inlineStr">
+        <is>
+          <t>Tier 5</t>
+        </is>
+      </c>
+      <c r="B46" s="80" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="C46" s="80" t="inlineStr">
+        <is>
+          <t>Group J</t>
+        </is>
+      </c>
+      <c r="D46" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="80" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F46" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="16" customHeight="1" s="28">
+      <c r="A47" s="80" t="inlineStr">
+        <is>
+          <t>Tier 5</t>
+        </is>
+      </c>
+      <c r="B47" s="80" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="C47" s="80" t="inlineStr">
+        <is>
+          <t>Group F</t>
+        </is>
+      </c>
+      <c r="D47" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="80" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F47" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1" s="28">
+      <c r="A48" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tier 6 – Major Underdogs</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="16" customHeight="1" s="28">
+      <c r="A49" s="84" t="inlineStr">
+        <is>
+          <t>Tier 6</t>
+        </is>
+      </c>
+      <c r="B49" s="84" t="inlineStr">
+        <is>
+          <t>Iraq</t>
+        </is>
+      </c>
+      <c r="C49" s="84" t="inlineStr">
+        <is>
+          <t>Group I</t>
+        </is>
+      </c>
+      <c r="D49" s="85" t="n">
+        <v>2</v>
+      </c>
+      <c r="E49" s="84" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="F49" s="86" t="inlineStr">
+        <is>
+          <t>Ryan Lowe, Peter Miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="16" customHeight="1" s="28">
+      <c r="A50" s="84" t="inlineStr">
+        <is>
+          <t>Tier 6</t>
+        </is>
+      </c>
+      <c r="B50" s="84" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="C50" s="84" t="inlineStr">
+        <is>
+          <t>Group L</t>
+        </is>
+      </c>
+      <c r="D50" s="85" t="n">
+        <v>2</v>
+      </c>
+      <c r="E50" s="84" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="F50" s="86" t="inlineStr">
+        <is>
+          <t>Ken Larade, Lucie Kendell</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="16" customHeight="1" s="28">
+      <c r="A51" s="84" t="inlineStr">
+        <is>
+          <t>Tier 6</t>
+        </is>
+      </c>
+      <c r="B51" s="84" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C51" s="84" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="D51" s="85" t="n">
+        <v>2</v>
+      </c>
+      <c r="E51" s="84" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="F51" s="86" t="inlineStr">
+        <is>
+          <t>Ken Larade, Ryan Lowe</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="16" customHeight="1" s="28">
+      <c r="A52" s="84" t="inlineStr">
+        <is>
+          <t>Tier 6</t>
+        </is>
+      </c>
+      <c r="B52" s="84" t="inlineStr">
+        <is>
+          <t>DR Congo</t>
+        </is>
+      </c>
+      <c r="C52" s="84" t="inlineStr">
+        <is>
+          <t>Group K</t>
+        </is>
+      </c>
+      <c r="D52" s="85" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="84" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F52" s="86" t="inlineStr">
+        <is>
+          <t>Lucie Kendell</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="16" customHeight="1" s="28">
+      <c r="A53" s="84" t="inlineStr">
+        <is>
+          <t>Tier 6</t>
+        </is>
+      </c>
+      <c r="B53" s="84" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="C53" s="84" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="D53" s="85" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="84" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F53" s="86" t="inlineStr">
+        <is>
+          <t>Peter Miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="16" customHeight="1" s="28">
+      <c r="A54" s="84" t="inlineStr">
+        <is>
+          <t>Tier 6</t>
+        </is>
+      </c>
+      <c r="B54" s="84" t="inlineStr">
+        <is>
+          <t>Cape Verde</t>
+        </is>
+      </c>
+      <c r="C54" s="84" t="inlineStr">
+        <is>
+          <t>Group H</t>
+        </is>
+      </c>
+      <c r="D54" s="84" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="84" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F54" s="86" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="16" customHeight="1" s="28">
+      <c r="A55" s="84" t="inlineStr">
+        <is>
+          <t>Tier 6</t>
+        </is>
+      </c>
+      <c r="B55" s="84" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+      <c r="C55" s="84" t="inlineStr">
+        <is>
+          <t>Group E</t>
+        </is>
+      </c>
+      <c r="D55" s="84" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="84" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F55" s="86" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="16" customHeight="1" s="28">
+      <c r="A56" s="84" t="inlineStr">
+        <is>
+          <t>Tier 6</t>
+        </is>
+      </c>
+      <c r="B56" s="84" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="C56" s="84" t="inlineStr">
+        <is>
+          <t>Group C</t>
+        </is>
+      </c>
+      <c r="D56" s="84" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="84" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F56" s="86" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A39:F39"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Rename Scoring tab to Picks; add pool analysis to Statistics tab
extract_picks.py / extract_scores.py:
- Tab renamed from "Scoring" to "Picks" across all scripts; old "Scoring"
  sheet removed automatically on next run

statistics.py / Statistics tab (4 new analyses):
  1. Consensus Lineup — most-picked team(s) per tier (ties included)
  2. Most Mainstream — participant whose picks have the highest overlap
     with the popular consensus (highest popularity score)
  3. Most Contrarian — participant whose picks most resemble the least-
     chosen teams (lowest popularity score)
  4. Uniqueness Score — per-participant 0–100 metric: average inverse-
     popularity of each pick ((1 - count/total) × 100 per team, averaged)

Results with current 4 submissions:
  Most mainstream: Peter Miles (popularity score 25)
  Most contrarian: Ryan Lowe  (popularity score 22, uniqueness 54.2%)

https://claude.ai/code/session_01VFqgqUhDsMbhjQyNveqHky
</commit_message>
<xml_diff>
--- a/WC2026_Pool.xlsx
+++ b/WC2026_Pool.xlsx
@@ -10,7 +10,7 @@
     <sheet name="User Submission Template" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Scoring Rules" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Entrants" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Scoring" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Picks" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Match Results" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Team Stats" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Statistics" sheetId="8" state="visible" r:id="rId8"/>
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="30">
+  <fonts count="37">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -208,8 +208,41 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007030A0"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007030A0"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="31">
+  <fills count="36">
     <fill>
       <patternFill/>
     </fill>
@@ -361,8 +394,33 @@
         <fgColor rgb="00E1E1E1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E4057"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8D5F5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -452,11 +510,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -704,6 +806,47 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="30" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="33" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="33" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="24" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4314,15 +4457,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" style="28" min="1" max="1"/>
-    <col width="20" customWidth="1" style="28" min="2" max="2"/>
+    <col width="22" customWidth="1" style="28" min="1" max="1"/>
+    <col width="12" customWidth="1" style="28" min="2" max="2"/>
     <col width="12" customWidth="1" style="28" min="3" max="3"/>
-    <col width="10" customWidth="1" style="28" min="4" max="4"/>
-    <col width="10" customWidth="1" style="28" min="5" max="5"/>
-    <col width="50" customWidth="1" style="28" min="6" max="6"/>
+    <col width="14" customWidth="1" style="28" min="4" max="4"/>
+    <col width="14" customWidth="1" style="28" min="5" max="5"/>
+    <col width="36" customWidth="1" style="28" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" s="28">
@@ -4333,32 +4476,32 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" s="28">
-      <c r="A2" s="61" t="inlineStr">
+      <c r="A2" s="49" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B2" s="61" t="inlineStr">
+      <c r="B2" s="49" t="inlineStr">
         <is>
           <t>Team</t>
         </is>
       </c>
-      <c r="C2" s="61" t="inlineStr">
+      <c r="C2" s="49" t="inlineStr">
         <is>
           <t>WC Group</t>
         </is>
       </c>
-      <c r="D2" s="61" t="inlineStr">
+      <c r="D2" s="49" t="inlineStr">
         <is>
           <t># Picked</t>
         </is>
       </c>
-      <c r="E2" s="61" t="inlineStr">
+      <c r="E2" s="49" t="inlineStr">
         <is>
           <t>% Picked</t>
         </is>
       </c>
-      <c r="F2" s="61" t="inlineStr">
+      <c r="F2" s="49" t="inlineStr">
         <is>
           <t>Picked By</t>
         </is>
@@ -5846,15 +5989,453 @@
         </is>
       </c>
     </row>
+    <row r="57" ht="8" customHeight="1" s="28"/>
+    <row r="58" ht="20" customHeight="1" s="28">
+      <c r="A58" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  POOL ANALYSIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="8" customHeight="1" s="28"/>
+    <row r="60" ht="20" customHeight="1" s="28">
+      <c r="A60" s="90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1.  Consensus Lineup  –  most popular pick(s) per tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1" s="28">
+      <c r="A61" s="91" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B61" s="91" t="inlineStr">
+        <is>
+          <t>Tier Description</t>
+        </is>
+      </c>
+      <c r="C61" s="91" t="inlineStr">
+        <is>
+          <t>Consensus Pick(s)</t>
+        </is>
+      </c>
+      <c r="D61" s="91" t="inlineStr">
+        <is>
+          <t>Times Picked</t>
+        </is>
+      </c>
+      <c r="E61" s="91" t="inlineStr">
+        <is>
+          <t>% of Pool</t>
+        </is>
+      </c>
+      <c r="F61" s="91" t="inlineStr"/>
+    </row>
+    <row r="62" ht="16" customHeight="1" s="28">
+      <c r="A62" s="92" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="B62" s="93" t="inlineStr">
+        <is>
+          <t>Elite Favorites</t>
+        </is>
+      </c>
+      <c r="C62" s="94" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D62" s="92" t="n">
+        <v>3</v>
+      </c>
+      <c r="E62" s="92" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="F62" s="92" t="inlineStr"/>
+    </row>
+    <row r="63" ht="16" customHeight="1" s="28">
+      <c r="A63" s="92" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="B63" s="93" t="inlineStr">
+        <is>
+          <t>Contenders</t>
+        </is>
+      </c>
+      <c r="C63" s="94" t="inlineStr">
+        <is>
+          <t>Belgium  /  Croatia  /  Morocco</t>
+        </is>
+      </c>
+      <c r="D63" s="92" t="n">
+        <v>2</v>
+      </c>
+      <c r="E63" s="92" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="F63" s="92" t="inlineStr"/>
+    </row>
+    <row r="64" ht="16" customHeight="1" s="28">
+      <c r="A64" s="92" t="inlineStr">
+        <is>
+          <t>Tier 3</t>
+        </is>
+      </c>
+      <c r="B64" s="93" t="inlineStr">
+        <is>
+          <t>Dark Horses</t>
+        </is>
+      </c>
+      <c r="C64" s="94" t="inlineStr">
+        <is>
+          <t>Norway  /  Switzerland</t>
+        </is>
+      </c>
+      <c r="D64" s="92" t="n">
+        <v>3</v>
+      </c>
+      <c r="E64" s="92" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="F64" s="92" t="inlineStr"/>
+    </row>
+    <row r="65" ht="16" customHeight="1" s="28">
+      <c r="A65" s="92" t="inlineStr">
+        <is>
+          <t>Tier 4</t>
+        </is>
+      </c>
+      <c r="B65" s="93" t="inlineStr">
+        <is>
+          <t>Long Shots</t>
+        </is>
+      </c>
+      <c r="C65" s="94" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="D65" s="92" t="n">
+        <v>3</v>
+      </c>
+      <c r="E65" s="92" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="F65" s="92" t="inlineStr"/>
+    </row>
+    <row r="66" ht="16" customHeight="1" s="28">
+      <c r="A66" s="92" t="inlineStr">
+        <is>
+          <t>Tier 5</t>
+        </is>
+      </c>
+      <c r="B66" s="93" t="inlineStr">
+        <is>
+          <t>Underdogs</t>
+        </is>
+      </c>
+      <c r="C66" s="94" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D66" s="92" t="n">
+        <v>3</v>
+      </c>
+      <c r="E66" s="92" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="F66" s="92" t="inlineStr"/>
+    </row>
+    <row r="67" ht="16" customHeight="1" s="28">
+      <c r="A67" s="92" t="inlineStr">
+        <is>
+          <t>Tier 6</t>
+        </is>
+      </c>
+      <c r="B67" s="93" t="inlineStr">
+        <is>
+          <t>Major Underdogs</t>
+        </is>
+      </c>
+      <c r="C67" s="94" t="inlineStr">
+        <is>
+          <t>Iraq  /  Panama  /  South Africa</t>
+        </is>
+      </c>
+      <c r="D67" s="92" t="n">
+        <v>2</v>
+      </c>
+      <c r="E67" s="92" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="F67" s="92" t="inlineStr"/>
+    </row>
+    <row r="68" ht="8" customHeight="1" s="28"/>
+    <row r="69" ht="20" customHeight="1" s="28">
+      <c r="A69" s="90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2 – 4.  Participant Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="14" customHeight="1" s="28">
+      <c r="A70" s="95" t="inlineStr">
+        <is>
+          <t>Popularity Score</t>
+        </is>
+      </c>
+      <c r="B70" s="96" t="inlineStr">
+        <is>
+          <t>Sum of how many participants picked each of your 12 teams (max = 48).  Higher = more mainstream.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="14" customHeight="1" s="28">
+      <c r="A71" s="95" t="inlineStr">
+        <is>
+          <t>Uniqueness Score</t>
+        </is>
+      </c>
+      <c r="B71" s="96" t="inlineStr">
+        <is>
+          <t>Average rarity of your picks, 0–100.  Per pick: (1 − pick_count ÷ 4) × 100.  Higher = more unique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="14" customHeight="1" s="28">
+      <c r="A72" s="95" t="inlineStr">
+        <is>
+          <t>Most Mainstream</t>
+        </is>
+      </c>
+      <c r="B72" s="96" t="inlineStr">
+        <is>
+          <t>Participant(s) with the highest popularity score — their picks most overlap the popular consensus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="14" customHeight="1" s="28">
+      <c r="A73" s="95" t="inlineStr">
+        <is>
+          <t>Most Contrarian</t>
+        </is>
+      </c>
+      <c r="B73" s="96" t="inlineStr">
+        <is>
+          <t>Participant(s) with the lowest popularity score — their picks most overlap the least-chosen teams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="8" customHeight="1" s="28"/>
+    <row r="75" ht="28" customHeight="1" s="28">
+      <c r="A75" s="91" t="inlineStr">
+        <is>
+          <t>Participant</t>
+        </is>
+      </c>
+      <c r="B75" s="91" t="inlineStr">
+        <is>
+          <t>Popularity
+Score</t>
+        </is>
+      </c>
+      <c r="C75" s="91" t="inlineStr">
+        <is>
+          <t>Uniqueness
+Score</t>
+        </is>
+      </c>
+      <c r="D75" s="91" t="inlineStr">
+        <is>
+          <t>Consensus
+Overlap</t>
+        </is>
+      </c>
+      <c r="E75" s="91" t="inlineStr">
+        <is>
+          <t>Contrarian
+Overlap</t>
+        </is>
+      </c>
+      <c r="F75" s="91" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="16" customHeight="1" s="28">
+      <c r="A76" s="94" t="inlineStr">
+        <is>
+          <t>Peter Miles</t>
+        </is>
+      </c>
+      <c r="B76" s="92" t="n">
+        <v>25</v>
+      </c>
+      <c r="C76" s="92" t="inlineStr">
+        <is>
+          <t>47.9</t>
+        </is>
+      </c>
+      <c r="D76" s="92" t="n">
+        <v>6</v>
+      </c>
+      <c r="E76" s="92" t="n">
+        <v>3</v>
+      </c>
+      <c r="F76" s="97" t="inlineStr">
+        <is>
+          <t>Most Mainstream</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="16" customHeight="1" s="28">
+      <c r="A77" s="59" t="inlineStr">
+        <is>
+          <t>Ken Larade</t>
+        </is>
+      </c>
+      <c r="B77" s="60" t="n">
+        <v>24</v>
+      </c>
+      <c r="C77" s="60" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="D77" s="60" t="n">
+        <v>7</v>
+      </c>
+      <c r="E77" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="F77" s="98" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="16" customHeight="1" s="28">
+      <c r="A78" s="94" t="inlineStr">
+        <is>
+          <t>Lucie Kendell</t>
+        </is>
+      </c>
+      <c r="B78" s="92" t="n">
+        <v>24</v>
+      </c>
+      <c r="C78" s="92" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="D78" s="92" t="n">
+        <v>7</v>
+      </c>
+      <c r="E78" s="92" t="n">
+        <v>3</v>
+      </c>
+      <c r="F78" s="93" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="16" customHeight="1" s="28">
+      <c r="A79" s="59" t="inlineStr">
+        <is>
+          <t>Ryan Lowe</t>
+        </is>
+      </c>
+      <c r="B79" s="60" t="n">
+        <v>22</v>
+      </c>
+      <c r="C79" s="60" t="inlineStr">
+        <is>
+          <t>54.2</t>
+        </is>
+      </c>
+      <c r="D79" s="60" t="n">
+        <v>7</v>
+      </c>
+      <c r="E79" s="60" t="n">
+        <v>5</v>
+      </c>
+      <c r="F79" s="99" t="inlineStr">
+        <is>
+          <t>Most Contrarian</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="8" customHeight="1" s="28"/>
+    <row r="81" ht="18" customHeight="1" s="28">
+      <c r="A81" s="100" t="inlineStr">
+        <is>
+          <t>Most like the popular consensus:</t>
+        </is>
+      </c>
+      <c r="D81" s="100" t="inlineStr">
+        <is>
+          <t>Peter Miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="18" customHeight="1" s="28">
+      <c r="A82" s="101" t="inlineStr">
+        <is>
+          <t>Most contrarian picks:</t>
+        </is>
+      </c>
+      <c r="D82" s="101" t="inlineStr">
+        <is>
+          <t>Ryan Lowe</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A1:F1"/>
+  <mergeCells count="23">
+    <mergeCell ref="B72:F72"/>
+    <mergeCell ref="A80:F80"/>
+    <mergeCell ref="A74:F74"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="B71:F71"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A21:F21"/>
+    <mergeCell ref="B70:F70"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="A81:C81"/>
+    <mergeCell ref="D82:F82"/>
+    <mergeCell ref="B73:F73"/>
+    <mergeCell ref="A68:F68"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A30:F30"/>
     <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="A82:C82"/>
+    <mergeCell ref="D81:F81"/>
+    <mergeCell ref="A60:F60"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A69:F69"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refresh WC2026_Pool.xlsx after script fixes
Regenerated by running extract_picks.py, extract_scores.py --mock, and
statistics.py following the path and constant fixes.

https://claude.ai/code/session_01VFqgqUhDsMbhjQyNveqHky
</commit_message>
<xml_diff>
--- a/WC2026_Pool.xlsx
+++ b/WC2026_Pool.xlsx
@@ -3019,7 +3019,7 @@
     <row r="3" ht="18" customHeight="1" s="28">
       <c r="A3" s="56" t="inlineStr">
         <is>
-          <t>Ken Larade</t>
+          <t>Ryan Lowe</t>
         </is>
       </c>
       <c r="B3" s="57" t="inlineStr">
@@ -3029,67 +3029,67 @@
       </c>
       <c r="C3" s="57" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="D3" s="57" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="E3" s="57" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="F3" s="57" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="G3" s="57" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="H3" s="57" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="I3" s="57" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="J3" s="57" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="K3" s="57" t="inlineStr">
         <is>
-          <t>Scotland</t>
+          <t>Uzbekistan</t>
         </is>
       </c>
       <c r="L3" s="57" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="M3" s="57" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="N3" s="58" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1" s="28">
       <c r="A4" s="59" t="inlineStr">
         <is>
-          <t>Ryan Lowe</t>
+          <t>Ken Larade</t>
         </is>
       </c>
       <c r="B4" s="60" t="inlineStr">
@@ -3099,61 +3099,61 @@
       </c>
       <c r="C4" s="60" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>France</t>
         </is>
       </c>
       <c r="D4" s="60" t="inlineStr">
         <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="E4" s="60" t="inlineStr">
+        <is>
           <t>Croatia</t>
         </is>
       </c>
-      <c r="E4" s="60" t="inlineStr">
-        <is>
-          <t>Morocco</t>
-        </is>
-      </c>
       <c r="F4" s="60" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="G4" s="60" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="H4" s="60" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="I4" s="60" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="J4" s="60" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="K4" s="60" t="inlineStr">
         <is>
-          <t>Uzbekistan</t>
+          <t>Scotland</t>
         </is>
       </c>
       <c r="L4" s="60" t="inlineStr">
         <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="M4" s="60" t="inlineStr">
+        <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="M4" s="60" t="inlineStr">
-        <is>
-          <t>Iraq</t>
-        </is>
-      </c>
       <c r="N4" s="58" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" s="28">

</xml_diff>

<commit_message>
Add fun badges to Statistics tab
Six awards computed and rendered in a new Awards & Badges section:

  ⭐ Crowd Favourite  – highest popularity score (most mainstream picks)
  🎯 Dark Horse       – highest uniqueness score (most contrarian picks)
  🐺 Lone Wolf        – most picks no one else made
  🌍 Globetrotter     – picks span the most different WC groups
  🎲 Group Gambler    – most picks concentrated in the same WC group
  🤝 Twins            – pair of participants with the most picks in common
                        (Jaccard similarity)

Also fixes a variable-shadowing bug: the consensus lineup loop used `teams`
as a loop variable, clobbering the `teams` function parameter before the
badges call — causing a ValueError when build_group_map tried to unpack
strings instead of 3-tuples. Renamed loop variable to `con_teams`.

https://claude.ai/code/session_01VFqgqUhDsMbhjQyNveqHky
</commit_message>
<xml_diff>
--- a/WC2026_Pool.xlsx
+++ b/WC2026_Pool.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="37">
+  <fonts count="49">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -241,8 +241,56 @@
       <color rgb="007030A0"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007F6000"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007F6000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="004A235A"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="004A235A"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000C343D"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="000C343D"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00274E13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00274E13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007F2B00"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007F2B00"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001C4587"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="001C4587"/>
+    </font>
   </fonts>
-  <fills count="36">
+  <fills count="42">
     <fill>
       <patternFill/>
     </fill>
@@ -419,6 +467,36 @@
         <fgColor rgb="00E8D5F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BF9000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAD1DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D0E0E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE5CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CFE2F3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="12">
     <border>
@@ -558,7 +636,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -847,6 +925,66 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="36" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="23" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="23" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="23" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="37" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="37" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="37" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="38" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="38" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="38" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="39" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="39" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="39" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="40" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="40" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="40" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="41" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="41" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="41" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4457,15 +4595,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="28" min="1" max="1"/>
-    <col width="12" customWidth="1" style="28" min="2" max="2"/>
-    <col width="12" customWidth="1" style="28" min="3" max="3"/>
-    <col width="14" customWidth="1" style="28" min="4" max="4"/>
-    <col width="14" customWidth="1" style="28" min="5" max="5"/>
-    <col width="36" customWidth="1" style="28" min="6" max="6"/>
+    <col width="28" customWidth="1" style="28" min="2" max="2"/>
+    <col width="5" customWidth="1" style="28" min="3" max="3"/>
+    <col width="22" customWidth="1" style="28" min="4" max="4"/>
+    <col width="5" customWidth="1" style="28" min="5" max="5"/>
+    <col width="52" customWidth="1" style="28" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" s="28">
@@ -6411,10 +6549,178 @@
         </is>
       </c>
     </row>
+    <row r="83" ht="8" customHeight="1" s="28"/>
+    <row r="84" ht="20" customHeight="1" s="28">
+      <c r="A84" s="102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AWARDS &amp; BADGES</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="18" customHeight="1" s="28">
+      <c r="A85" s="103" t="inlineStr">
+        <is>
+          <t>Badge</t>
+        </is>
+      </c>
+      <c r="B85" s="103" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+      <c r="C85" s="103" t="inlineStr"/>
+      <c r="D85" s="103" t="inlineStr">
+        <is>
+          <t>Winner(s)</t>
+        </is>
+      </c>
+      <c r="E85" s="103" t="inlineStr"/>
+      <c r="F85" s="103" t="inlineStr">
+        <is>
+          <t>Earning stat</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1" s="28">
+      <c r="A86" s="104" t="inlineStr">
+        <is>
+          <t>⭐  Crowd Favourite</t>
+        </is>
+      </c>
+      <c r="B86" s="105" t="inlineStr">
+        <is>
+          <t>Most mainstream picks — highest overlap with the popular consensus</t>
+        </is>
+      </c>
+      <c r="D86" s="104" t="inlineStr">
+        <is>
+          <t>Peter Miles</t>
+        </is>
+      </c>
+      <c r="F86" s="106" t="inlineStr">
+        <is>
+          <t>Popularity score: 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1" s="28">
+      <c r="A87" s="107" t="inlineStr">
+        <is>
+          <t>🎯  Dark Horse</t>
+        </is>
+      </c>
+      <c r="B87" s="108" t="inlineStr">
+        <is>
+          <t>Most contrarian picks — highest uniqueness score</t>
+        </is>
+      </c>
+      <c r="D87" s="107" t="inlineStr">
+        <is>
+          <t>Ryan Lowe</t>
+        </is>
+      </c>
+      <c r="F87" s="109" t="inlineStr">
+        <is>
+          <t>Uniqueness: 54.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1" s="28">
+      <c r="A88" s="110" t="inlineStr">
+        <is>
+          <t>🐺  Lone Wolf</t>
+        </is>
+      </c>
+      <c r="B88" s="111" t="inlineStr">
+        <is>
+          <t>Most picks that nobody else made</t>
+        </is>
+      </c>
+      <c r="D88" s="110" t="inlineStr">
+        <is>
+          <t>Ryan Lowe</t>
+        </is>
+      </c>
+      <c r="F88" s="112" t="inlineStr">
+        <is>
+          <t>5 exclusive pick(s): Argentina, Australia, Ecuador, New Zealand, Uzbekistan</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="22" customHeight="1" s="28">
+      <c r="A89" s="113" t="inlineStr">
+        <is>
+          <t>🌍  Globetrotter</t>
+        </is>
+      </c>
+      <c r="B89" s="114" t="inlineStr">
+        <is>
+          <t>Picks span the most different WC groups</t>
+        </is>
+      </c>
+      <c r="D89" s="113" t="inlineStr">
+        <is>
+          <t>Ryan Lowe</t>
+        </is>
+      </c>
+      <c r="F89" s="115" t="inlineStr">
+        <is>
+          <t>12 different WC groups covered</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="22" customHeight="1" s="28">
+      <c r="A90" s="116" t="inlineStr">
+        <is>
+          <t>🎲  Group Gambler</t>
+        </is>
+      </c>
+      <c r="B90" s="117" t="inlineStr">
+        <is>
+          <t>Most picks from the same WC group — highest concentration risk</t>
+        </is>
+      </c>
+      <c r="D90" s="116" t="inlineStr">
+        <is>
+          <t>Ken Larade  /  Peter Miles</t>
+        </is>
+      </c>
+      <c r="F90" s="118" t="inlineStr">
+        <is>
+          <t>3 picks from Group I / Group L: Croatia, France, Ghana, Iraq, Norway, Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1" s="28">
+      <c r="A91" s="119" t="inlineStr">
+        <is>
+          <t>🤝  Twins</t>
+        </is>
+      </c>
+      <c r="B91" s="120" t="inlineStr">
+        <is>
+          <t>The pair of participants with the most picks in common</t>
+        </is>
+      </c>
+      <c r="D91" s="119" t="inlineStr">
+        <is>
+          <t>Ken Larade &amp; Lucie Kendell</t>
+        </is>
+      </c>
+      <c r="F91" s="121" t="inlineStr">
+        <is>
+          <t>5 shared picks (26% similarity): Belgium, Canada, Norway, Panama, Spain</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="37">
+    <mergeCell ref="B91:C91"/>
+    <mergeCell ref="A84:F84"/>
+    <mergeCell ref="B90:C90"/>
     <mergeCell ref="B72:F72"/>
     <mergeCell ref="A80:F80"/>
+    <mergeCell ref="D90:E90"/>
     <mergeCell ref="A74:F74"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="B71:F71"/>
@@ -6422,11 +6728,18 @@
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="B70:F70"/>
     <mergeCell ref="A57:F57"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="D86:E86"/>
+    <mergeCell ref="B88:C88"/>
     <mergeCell ref="A81:C81"/>
+    <mergeCell ref="D91:E91"/>
     <mergeCell ref="D82:F82"/>
     <mergeCell ref="B73:F73"/>
+    <mergeCell ref="B87:C87"/>
+    <mergeCell ref="D87:E87"/>
     <mergeCell ref="A68:F68"/>
     <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A83:F83"/>
     <mergeCell ref="A48:F48"/>
     <mergeCell ref="A30:F30"/>
     <mergeCell ref="A39:F39"/>
@@ -6435,6 +6748,9 @@
     <mergeCell ref="D81:F81"/>
     <mergeCell ref="A60:F60"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B89:C89"/>
+    <mergeCell ref="D89:E89"/>
+    <mergeCell ref="D88:E88"/>
     <mergeCell ref="A69:F69"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add update_scoring.py with Scores and Scoring tabs
Creates two new tabs in WC2026_Pool.xlsx:
- Scores: all 72 group stage matchups pre-populated (Groups A-L) plus
  32 knockout placeholder rows; score cells highlighted yellow for easy entry.
- Scoring: leaderboard ranked by total points + per-pick breakdown
  with tier-coloured columns; recomputes automatically from finished
  rows in the Scores tab using pool scoring rules (match pts + group bonuses).

https://claude.ai/code/session_01VFqgqUhDsMbhjQyNveqHky
</commit_message>
<xml_diff>
--- a/WC2026_Pool.xlsx
+++ b/WC2026_Pool.xlsx
@@ -14,6 +14,8 @@
     <sheet name="Match Results" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Team Stats" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Statistics" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Scores" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Scoring" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -23,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="49">
+  <fonts count="52">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -289,8 +291,16 @@
       <i val="1"/>
       <color rgb="001C4587"/>
     </font>
+    <font>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font/>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="42">
+  <fills count="50">
     <fill>
       <patternFill/>
     </fill>
@@ -497,6 +507,46 @@
         <fgColor rgb="00CFE2F3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00243F60"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD700"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="12">
     <border>
@@ -636,7 +686,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="161">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -986,6 +1036,123 @@
     </xf>
     <xf numFmtId="0" fontId="48" fillId="41" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="42" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="43" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="43" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="44" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="39" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="41" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="41" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="45" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="45" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="46" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="47" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="47" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="38" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="49" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="49" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="49" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="16" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="24" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="19" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="20" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="21" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="43" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="22" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2294,6 +2461,750 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" style="28" min="1" max="1"/>
+    <col width="22" customWidth="1" style="28" min="2" max="2"/>
+    <col width="14" customWidth="1" style="28" min="3" max="3"/>
+    <col width="16" customWidth="1" style="28" min="4" max="4"/>
+    <col width="16" customWidth="1" style="28" min="5" max="5"/>
+    <col width="16" customWidth="1" style="28" min="6" max="6"/>
+    <col width="7" customWidth="1" style="28" min="7" max="7"/>
+    <col width="16" customWidth="1" style="28" min="8" max="8"/>
+    <col width="7" customWidth="1" style="28" min="9" max="9"/>
+    <col width="16" customWidth="1" style="28" min="10" max="10"/>
+    <col width="7" customWidth="1" style="28" min="11" max="11"/>
+    <col width="16" customWidth="1" style="28" min="12" max="12"/>
+    <col width="7" customWidth="1" style="28" min="13" max="13"/>
+    <col width="16" customWidth="1" style="28" min="14" max="14"/>
+    <col width="7" customWidth="1" style="28" min="15" max="15"/>
+    <col width="16" customWidth="1" style="28" min="16" max="16"/>
+    <col width="7" customWidth="1" style="28" min="17" max="17"/>
+    <col width="16" customWidth="1" style="28" min="18" max="18"/>
+    <col width="7" customWidth="1" style="28" min="19" max="19"/>
+    <col width="16" customWidth="1" style="28" min="20" max="20"/>
+    <col width="7" customWidth="1" style="28" min="21" max="21"/>
+    <col width="16" customWidth="1" style="28" min="22" max="22"/>
+    <col width="7" customWidth="1" style="28" min="23" max="23"/>
+    <col width="16" customWidth="1" style="28" min="24" max="24"/>
+    <col width="7" customWidth="1" style="28" min="25" max="25"/>
+    <col width="7" customWidth="1" style="28" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1" s="28">
+      <c r="A1" s="48" t="inlineStr">
+        <is>
+          <t>2026 FIFA World Cup Pool – Scoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="28">
+      <c r="A2" s="144" t="inlineStr">
+        <is>
+          <t>LEADERBOARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="28">
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B3" s="61" t="inlineStr">
+        <is>
+          <t>Participant</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="inlineStr">
+        <is>
+          <t>Total Points</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>Pts from Matches</t>
+        </is>
+      </c>
+      <c r="E3" s="61" t="inlineStr">
+        <is>
+          <t>Pts from Bonuses</t>
+        </is>
+      </c>
+      <c r="F3" s="61" t="inlineStr">
+        <is>
+          <t># Scored Teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="146" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="147" t="inlineStr">
+        <is>
+          <t>Ryan Lowe</t>
+        </is>
+      </c>
+      <c r="C4" s="146" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="148" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="149" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="150" t="inlineStr">
+        <is>
+          <t>Ken Larade</t>
+        </is>
+      </c>
+      <c r="C5" s="149" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="151" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="98" t="inlineStr">
+        <is>
+          <t>Lucie Kendell</t>
+        </is>
+      </c>
+      <c r="C6" s="151" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="149" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="150" t="inlineStr">
+        <is>
+          <t>Peter Miles</t>
+        </is>
+      </c>
+      <c r="C7" s="149" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" s="28">
+      <c r="A9" s="144" t="inlineStr">
+        <is>
+          <t>PICKS BREAKDOWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" s="28">
+      <c r="A10" s="49" t="inlineStr">
+        <is>
+          <t>Participant</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>T1 Pick 1</t>
+        </is>
+      </c>
+      <c r="C10" s="49" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="D10" s="49" t="inlineStr">
+        <is>
+          <t>T1 Pick 2</t>
+        </is>
+      </c>
+      <c r="E10" s="49" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="F10" s="49" t="inlineStr">
+        <is>
+          <t>T2 Pick 1</t>
+        </is>
+      </c>
+      <c r="G10" s="49" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="H10" s="49" t="inlineStr">
+        <is>
+          <t>T2 Pick 2</t>
+        </is>
+      </c>
+      <c r="I10" s="49" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="J10" s="49" t="inlineStr">
+        <is>
+          <t>T3 Pick 1</t>
+        </is>
+      </c>
+      <c r="K10" s="49" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="L10" s="49" t="inlineStr">
+        <is>
+          <t>T3 Pick 2</t>
+        </is>
+      </c>
+      <c r="M10" s="49" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="N10" s="49" t="inlineStr">
+        <is>
+          <t>T4 Pick 1</t>
+        </is>
+      </c>
+      <c r="O10" s="49" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="P10" s="49" t="inlineStr">
+        <is>
+          <t>T4 Pick 2</t>
+        </is>
+      </c>
+      <c r="Q10" s="49" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="R10" s="49" t="inlineStr">
+        <is>
+          <t>T5 Pick 1</t>
+        </is>
+      </c>
+      <c r="S10" s="49" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="T10" s="49" t="inlineStr">
+        <is>
+          <t>T5 Pick 2</t>
+        </is>
+      </c>
+      <c r="U10" s="49" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="V10" s="49" t="inlineStr">
+        <is>
+          <t>T6 Pick 1</t>
+        </is>
+      </c>
+      <c r="W10" s="49" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="X10" s="49" t="inlineStr">
+        <is>
+          <t>T6 Pick 2</t>
+        </is>
+      </c>
+      <c r="Y10" s="49" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="Z10" s="49" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="59" t="inlineStr">
+        <is>
+          <t>Ryan Lowe</t>
+        </is>
+      </c>
+      <c r="B11" s="152" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C11" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="152" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E11" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="154" t="inlineStr">
+        <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="G11" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="154" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="I11" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="155" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="K11" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="155" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="M11" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="156" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="O11" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="156" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="Q11" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="157" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="S11" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="157" t="inlineStr">
+        <is>
+          <t>Uzbekistan</t>
+        </is>
+      </c>
+      <c r="U11" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="158" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="W11" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="158" t="inlineStr">
+        <is>
+          <t>Iraq</t>
+        </is>
+      </c>
+      <c r="Y11" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="56" t="inlineStr">
+        <is>
+          <t>Ken Larade</t>
+        </is>
+      </c>
+      <c r="B12" s="152" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C12" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="152" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="E12" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="154" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="G12" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="154" t="inlineStr">
+        <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="I12" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="155" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="K12" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="155" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="M12" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="156" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="O12" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="156" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="Q12" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="157" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="S12" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="157" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="U12" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" s="158" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="W12" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" s="158" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="Y12" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="59" t="inlineStr">
+        <is>
+          <t>Lucie Kendell</t>
+        </is>
+      </c>
+      <c r="B13" s="152" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C13" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="152" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="E13" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="154" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="G13" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="154" t="inlineStr">
+        <is>
+          <t>Columbia</t>
+        </is>
+      </c>
+      <c r="I13" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="155" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="K13" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="155" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="M13" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="156" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="O13" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="156" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="Q13" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="157" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="S13" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="157" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="U13" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="158" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="W13" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="158" t="inlineStr">
+        <is>
+          <t>DR Congo</t>
+        </is>
+      </c>
+      <c r="Y13" s="153" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="56" t="inlineStr">
+        <is>
+          <t>Peter Miles</t>
+        </is>
+      </c>
+      <c r="B14" s="152" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C14" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="152" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E14" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="154" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="G14" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="154" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="I14" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="155" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="K14" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="155" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="M14" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="156" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="O14" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="156" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="Q14" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="157" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="S14" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="157" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="U14" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="158" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="W14" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="158" t="inlineStr">
+        <is>
+          <t>Iraq</t>
+        </is>
+      </c>
+      <c r="Y14" s="160" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A9:F9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4651,6 +5562,11 @@
           <t xml:space="preserve">  Tier 1 – Elite Favorites</t>
         </is>
       </c>
+      <c r="B3" s="87" t="n"/>
+      <c r="C3" s="87" t="n"/>
+      <c r="D3" s="87" t="n"/>
+      <c r="E3" s="87" t="n"/>
+      <c r="F3" s="88" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1" s="28">
       <c r="A4" s="64" t="inlineStr">
@@ -4898,6 +5814,11 @@
           <t xml:space="preserve">  Tier 2 – Contenders</t>
         </is>
       </c>
+      <c r="B12" s="87" t="n"/>
+      <c r="C12" s="87" t="n"/>
+      <c r="D12" s="87" t="n"/>
+      <c r="E12" s="87" t="n"/>
+      <c r="F12" s="88" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1" s="28">
       <c r="A13" s="68" t="inlineStr">
@@ -5145,6 +6066,11 @@
           <t xml:space="preserve">  Tier 3 – Dark Horses</t>
         </is>
       </c>
+      <c r="B21" s="87" t="n"/>
+      <c r="C21" s="87" t="n"/>
+      <c r="D21" s="87" t="n"/>
+      <c r="E21" s="87" t="n"/>
+      <c r="F21" s="88" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1" s="28">
       <c r="A22" s="72" t="inlineStr">
@@ -5392,6 +6318,11 @@
           <t xml:space="preserve">  Tier 4 – Long Shots</t>
         </is>
       </c>
+      <c r="B30" s="87" t="n"/>
+      <c r="C30" s="87" t="n"/>
+      <c r="D30" s="87" t="n"/>
+      <c r="E30" s="87" t="n"/>
+      <c r="F30" s="88" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1" s="28">
       <c r="A31" s="76" t="inlineStr">
@@ -5639,6 +6570,11 @@
           <t xml:space="preserve">  Tier 5 – Underdogs</t>
         </is>
       </c>
+      <c r="B39" s="87" t="n"/>
+      <c r="C39" s="87" t="n"/>
+      <c r="D39" s="87" t="n"/>
+      <c r="E39" s="87" t="n"/>
+      <c r="F39" s="88" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1" s="28">
       <c r="A40" s="80" t="inlineStr">
@@ -5886,6 +6822,11 @@
           <t xml:space="preserve">  Tier 6 – Major Underdogs</t>
         </is>
       </c>
+      <c r="B48" s="87" t="n"/>
+      <c r="C48" s="87" t="n"/>
+      <c r="D48" s="87" t="n"/>
+      <c r="E48" s="87" t="n"/>
+      <c r="F48" s="88" t="n"/>
     </row>
     <row r="49" ht="16" customHeight="1" s="28">
       <c r="A49" s="84" t="inlineStr">
@@ -6592,11 +7533,13 @@
           <t>Most mainstream picks — highest overlap with the popular consensus</t>
         </is>
       </c>
+      <c r="C86" s="88" t="n"/>
       <c r="D86" s="104" t="inlineStr">
         <is>
           <t>Peter Miles</t>
         </is>
       </c>
+      <c r="E86" s="88" t="n"/>
       <c r="F86" s="106" t="inlineStr">
         <is>
           <t>Popularity score: 25</t>
@@ -6614,11 +7557,13 @@
           <t>Most contrarian picks — highest uniqueness score</t>
         </is>
       </c>
+      <c r="C87" s="88" t="n"/>
       <c r="D87" s="107" t="inlineStr">
         <is>
           <t>Ryan Lowe</t>
         </is>
       </c>
+      <c r="E87" s="88" t="n"/>
       <c r="F87" s="109" t="inlineStr">
         <is>
           <t>Uniqueness: 54.2%</t>
@@ -6636,11 +7581,13 @@
           <t>Most picks that nobody else made</t>
         </is>
       </c>
+      <c r="C88" s="88" t="n"/>
       <c r="D88" s="110" t="inlineStr">
         <is>
           <t>Ryan Lowe</t>
         </is>
       </c>
+      <c r="E88" s="88" t="n"/>
       <c r="F88" s="112" t="inlineStr">
         <is>
           <t>5 exclusive pick(s): Argentina, Australia, Ecuador, New Zealand, Uzbekistan</t>
@@ -6658,11 +7605,13 @@
           <t>Picks span the most different WC groups</t>
         </is>
       </c>
+      <c r="C89" s="88" t="n"/>
       <c r="D89" s="113" t="inlineStr">
         <is>
           <t>Ryan Lowe</t>
         </is>
       </c>
+      <c r="E89" s="88" t="n"/>
       <c r="F89" s="115" t="inlineStr">
         <is>
           <t>12 different WC groups covered</t>
@@ -6680,11 +7629,13 @@
           <t>Most picks from the same WC group — highest concentration risk</t>
         </is>
       </c>
+      <c r="C90" s="88" t="n"/>
       <c r="D90" s="116" t="inlineStr">
         <is>
           <t>Ken Larade  /  Peter Miles</t>
         </is>
       </c>
+      <c r="E90" s="88" t="n"/>
       <c r="F90" s="118" t="inlineStr">
         <is>
           <t>3 picks from Group I / Group L: Croatia, France, Ghana, Iraq, Norway, Panama</t>
@@ -6702,11 +7653,13 @@
           <t>The pair of participants with the most picks in common</t>
         </is>
       </c>
+      <c r="C91" s="88" t="n"/>
       <c r="D91" s="119" t="inlineStr">
         <is>
           <t>Ken Larade &amp; Lucie Kendell</t>
         </is>
       </c>
+      <c r="E91" s="88" t="n"/>
       <c r="F91" s="121" t="inlineStr">
         <is>
           <t>5 shared picks (26% similarity): Belgium, Canada, Norway, Panama, Spain</t>
@@ -6718,8 +7671,8 @@
     <mergeCell ref="B91:C91"/>
     <mergeCell ref="A84:F84"/>
     <mergeCell ref="B90:C90"/>
+    <mergeCell ref="A80:F80"/>
     <mergeCell ref="B72:F72"/>
-    <mergeCell ref="A80:F80"/>
     <mergeCell ref="D90:E90"/>
     <mergeCell ref="A74:F74"/>
     <mergeCell ref="A12:F12"/>
@@ -6755,4 +7708,3413 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J142"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" style="28" min="1" max="1"/>
+    <col width="16" customWidth="1" style="28" min="2" max="2"/>
+    <col width="8" customWidth="1" style="28" min="3" max="3"/>
+    <col width="16" customWidth="1" style="28" min="4" max="4"/>
+    <col width="20" customWidth="1" style="28" min="5" max="5"/>
+    <col width="12" customWidth="1" style="28" min="6" max="6"/>
+    <col width="12" customWidth="1" style="28" min="7" max="7"/>
+    <col width="20" customWidth="1" style="28" min="8" max="8"/>
+    <col width="16" customWidth="1" style="28" min="9" max="9"/>
+    <col width="24" customWidth="1" style="28" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1" s="28">
+      <c r="A1" s="48" t="inlineStr">
+        <is>
+          <t>2026 FIFA World Cup – Match Scores</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1" s="28">
+      <c r="A2" s="61" t="inlineStr">
+        <is>
+          <t>Match #</t>
+        </is>
+      </c>
+      <c r="B2" s="61" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C2" s="61" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D2" s="61" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="E2" s="61" t="inlineStr">
+        <is>
+          <t>Home Team</t>
+        </is>
+      </c>
+      <c r="F2" s="61" t="inlineStr">
+        <is>
+          <t>Home Score</t>
+        </is>
+      </c>
+      <c r="G2" s="61" t="inlineStr">
+        <is>
+          <t>Away Score</t>
+        </is>
+      </c>
+      <c r="H2" s="61" t="inlineStr">
+        <is>
+          <t>Away Team</t>
+        </is>
+      </c>
+      <c r="I2" s="61" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="J2" s="61" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1" s="28">
+      <c r="A3" s="122" t="inlineStr">
+        <is>
+          <t>Group A  –  Mexico | South Korea | South Africa | Czechia</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1" s="28">
+      <c r="A4" s="123" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="123" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C4" s="123" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="D4" s="123" t="inlineStr"/>
+      <c r="E4" s="123" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="F4" s="58" t="n"/>
+      <c r="G4" s="58" t="n"/>
+      <c r="H4" s="123" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="I4" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J4" s="123" t="inlineStr"/>
+    </row>
+    <row r="5" ht="16" customHeight="1" s="28">
+      <c r="A5" s="123" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="123" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C5" s="123" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="D5" s="123" t="inlineStr"/>
+      <c r="E5" s="123" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="F5" s="58" t="n"/>
+      <c r="G5" s="58" t="n"/>
+      <c r="H5" s="123" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I5" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J5" s="123" t="inlineStr"/>
+    </row>
+    <row r="6" ht="16" customHeight="1" s="28">
+      <c r="A6" s="123" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="123" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C6" s="123" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="D6" s="123" t="inlineStr"/>
+      <c r="E6" s="123" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="F6" s="58" t="n"/>
+      <c r="G6" s="58" t="n"/>
+      <c r="H6" s="123" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="I6" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J6" s="123" t="inlineStr"/>
+    </row>
+    <row r="7" ht="16" customHeight="1" s="28">
+      <c r="A7" s="123" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="123" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C7" s="123" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="D7" s="123" t="inlineStr"/>
+      <c r="E7" s="123" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="F7" s="58" t="n"/>
+      <c r="G7" s="58" t="n"/>
+      <c r="H7" s="123" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I7" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J7" s="123" t="inlineStr"/>
+    </row>
+    <row r="8" ht="16" customHeight="1" s="28">
+      <c r="A8" s="123" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="123" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C8" s="123" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="D8" s="123" t="inlineStr"/>
+      <c r="E8" s="123" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="F8" s="58" t="n"/>
+      <c r="G8" s="58" t="n"/>
+      <c r="H8" s="123" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="I8" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J8" s="123" t="inlineStr"/>
+    </row>
+    <row r="9" ht="16" customHeight="1" s="28">
+      <c r="A9" s="123" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="123" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C9" s="123" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="D9" s="123" t="inlineStr"/>
+      <c r="E9" s="123" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="F9" s="58" t="n"/>
+      <c r="G9" s="58" t="n"/>
+      <c r="H9" s="123" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="I9" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J9" s="123" t="inlineStr"/>
+    </row>
+    <row r="10"/>
+    <row r="11" ht="18" customHeight="1" s="28">
+      <c r="A11" s="124" t="inlineStr">
+        <is>
+          <t>Group B  –  Canada | Switzerland | Bosnia &amp; Herz. | Qatar</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1" s="28">
+      <c r="A12" s="125" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="125" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C12" s="125" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="D12" s="125" t="inlineStr"/>
+      <c r="E12" s="125" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F12" s="58" t="n"/>
+      <c r="G12" s="58" t="n"/>
+      <c r="H12" s="125" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="I12" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J12" s="125" t="inlineStr"/>
+    </row>
+    <row r="13" ht="16" customHeight="1" s="28">
+      <c r="A13" s="125" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="125" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C13" s="125" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="D13" s="125" t="inlineStr"/>
+      <c r="E13" s="125" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F13" s="58" t="n"/>
+      <c r="G13" s="58" t="n"/>
+      <c r="H13" s="125" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herz.</t>
+        </is>
+      </c>
+      <c r="I13" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J13" s="125" t="inlineStr"/>
+    </row>
+    <row r="14" ht="16" customHeight="1" s="28">
+      <c r="A14" s="125" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="125" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C14" s="125" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="D14" s="125" t="inlineStr"/>
+      <c r="E14" s="125" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F14" s="58" t="n"/>
+      <c r="G14" s="58" t="n"/>
+      <c r="H14" s="125" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="I14" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J14" s="125" t="inlineStr"/>
+    </row>
+    <row r="15" ht="16" customHeight="1" s="28">
+      <c r="A15" s="125" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="125" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C15" s="125" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="D15" s="125" t="inlineStr"/>
+      <c r="E15" s="125" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="F15" s="58" t="n"/>
+      <c r="G15" s="58" t="n"/>
+      <c r="H15" s="125" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herz.</t>
+        </is>
+      </c>
+      <c r="I15" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J15" s="125" t="inlineStr"/>
+    </row>
+    <row r="16" ht="16" customHeight="1" s="28">
+      <c r="A16" s="125" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="125" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C16" s="125" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="D16" s="125" t="inlineStr"/>
+      <c r="E16" s="125" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="F16" s="58" t="n"/>
+      <c r="G16" s="58" t="n"/>
+      <c r="H16" s="125" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="I16" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J16" s="125" t="inlineStr"/>
+    </row>
+    <row r="17" ht="16" customHeight="1" s="28">
+      <c r="A17" s="125" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="125" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C17" s="125" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="D17" s="125" t="inlineStr"/>
+      <c r="E17" s="125" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herz.</t>
+        </is>
+      </c>
+      <c r="F17" s="58" t="n"/>
+      <c r="G17" s="58" t="n"/>
+      <c r="H17" s="125" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="I17" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J17" s="125" t="inlineStr"/>
+    </row>
+    <row r="18"/>
+    <row r="19" ht="18" customHeight="1" s="28">
+      <c r="A19" s="126" t="inlineStr">
+        <is>
+          <t>Group C  –  Brazil | Morocco | Scotland | Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1" s="28">
+      <c r="A20" s="127" t="n">
+        <v>13</v>
+      </c>
+      <c r="B20" s="127" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C20" s="127" t="inlineStr">
+        <is>
+          <t>Group C</t>
+        </is>
+      </c>
+      <c r="D20" s="127" t="inlineStr"/>
+      <c r="E20" s="127" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="F20" s="58" t="n"/>
+      <c r="G20" s="58" t="n"/>
+      <c r="H20" s="127" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="I20" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J20" s="127" t="inlineStr"/>
+    </row>
+    <row r="21" ht="16" customHeight="1" s="28">
+      <c r="A21" s="127" t="n">
+        <v>14</v>
+      </c>
+      <c r="B21" s="127" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C21" s="127" t="inlineStr">
+        <is>
+          <t>Group C</t>
+        </is>
+      </c>
+      <c r="D21" s="127" t="inlineStr"/>
+      <c r="E21" s="127" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="F21" s="58" t="n"/>
+      <c r="G21" s="58" t="n"/>
+      <c r="H21" s="127" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="I21" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J21" s="127" t="inlineStr"/>
+    </row>
+    <row r="22" ht="16" customHeight="1" s="28">
+      <c r="A22" s="127" t="n">
+        <v>15</v>
+      </c>
+      <c r="B22" s="127" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C22" s="127" t="inlineStr">
+        <is>
+          <t>Group C</t>
+        </is>
+      </c>
+      <c r="D22" s="127" t="inlineStr"/>
+      <c r="E22" s="127" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="F22" s="58" t="n"/>
+      <c r="G22" s="58" t="n"/>
+      <c r="H22" s="127" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="I22" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J22" s="127" t="inlineStr"/>
+    </row>
+    <row r="23" ht="16" customHeight="1" s="28">
+      <c r="A23" s="127" t="n">
+        <v>16</v>
+      </c>
+      <c r="B23" s="127" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C23" s="127" t="inlineStr">
+        <is>
+          <t>Group C</t>
+        </is>
+      </c>
+      <c r="D23" s="127" t="inlineStr"/>
+      <c r="E23" s="127" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="F23" s="58" t="n"/>
+      <c r="G23" s="58" t="n"/>
+      <c r="H23" s="127" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="I23" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J23" s="127" t="inlineStr"/>
+    </row>
+    <row r="24" ht="16" customHeight="1" s="28">
+      <c r="A24" s="127" t="n">
+        <v>17</v>
+      </c>
+      <c r="B24" s="127" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C24" s="127" t="inlineStr">
+        <is>
+          <t>Group C</t>
+        </is>
+      </c>
+      <c r="D24" s="127" t="inlineStr"/>
+      <c r="E24" s="127" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="F24" s="58" t="n"/>
+      <c r="G24" s="58" t="n"/>
+      <c r="H24" s="127" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="I24" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J24" s="127" t="inlineStr"/>
+    </row>
+    <row r="25" ht="16" customHeight="1" s="28">
+      <c r="A25" s="127" t="n">
+        <v>18</v>
+      </c>
+      <c r="B25" s="127" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C25" s="127" t="inlineStr">
+        <is>
+          <t>Group C</t>
+        </is>
+      </c>
+      <c r="D25" s="127" t="inlineStr"/>
+      <c r="E25" s="127" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="F25" s="58" t="n"/>
+      <c r="G25" s="58" t="n"/>
+      <c r="H25" s="127" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="I25" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J25" s="127" t="inlineStr"/>
+    </row>
+    <row r="26"/>
+    <row r="27" ht="18" customHeight="1" s="28">
+      <c r="A27" s="128" t="inlineStr">
+        <is>
+          <t>Group D  –  United States | Turkey | Australia | Paraguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1" s="28">
+      <c r="A28" s="129" t="n">
+        <v>19</v>
+      </c>
+      <c r="B28" s="129" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C28" s="129" t="inlineStr">
+        <is>
+          <t>Group D</t>
+        </is>
+      </c>
+      <c r="D28" s="129" t="inlineStr"/>
+      <c r="E28" s="129" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F28" s="58" t="n"/>
+      <c r="G28" s="58" t="n"/>
+      <c r="H28" s="129" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="I28" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J28" s="129" t="inlineStr"/>
+    </row>
+    <row r="29" ht="16" customHeight="1" s="28">
+      <c r="A29" s="129" t="n">
+        <v>20</v>
+      </c>
+      <c r="B29" s="129" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C29" s="129" t="inlineStr">
+        <is>
+          <t>Group D</t>
+        </is>
+      </c>
+      <c r="D29" s="129" t="inlineStr"/>
+      <c r="E29" s="129" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F29" s="58" t="n"/>
+      <c r="G29" s="58" t="n"/>
+      <c r="H29" s="129" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="I29" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J29" s="129" t="inlineStr"/>
+    </row>
+    <row r="30" ht="16" customHeight="1" s="28">
+      <c r="A30" s="129" t="n">
+        <v>21</v>
+      </c>
+      <c r="B30" s="129" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C30" s="129" t="inlineStr">
+        <is>
+          <t>Group D</t>
+        </is>
+      </c>
+      <c r="D30" s="129" t="inlineStr"/>
+      <c r="E30" s="129" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F30" s="58" t="n"/>
+      <c r="G30" s="58" t="n"/>
+      <c r="H30" s="129" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="I30" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J30" s="129" t="inlineStr"/>
+    </row>
+    <row r="31" ht="16" customHeight="1" s="28">
+      <c r="A31" s="129" t="n">
+        <v>22</v>
+      </c>
+      <c r="B31" s="129" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C31" s="129" t="inlineStr">
+        <is>
+          <t>Group D</t>
+        </is>
+      </c>
+      <c r="D31" s="129" t="inlineStr"/>
+      <c r="E31" s="129" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="F31" s="58" t="n"/>
+      <c r="G31" s="58" t="n"/>
+      <c r="H31" s="129" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="I31" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J31" s="129" t="inlineStr"/>
+    </row>
+    <row r="32" ht="16" customHeight="1" s="28">
+      <c r="A32" s="129" t="n">
+        <v>23</v>
+      </c>
+      <c r="B32" s="129" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C32" s="129" t="inlineStr">
+        <is>
+          <t>Group D</t>
+        </is>
+      </c>
+      <c r="D32" s="129" t="inlineStr"/>
+      <c r="E32" s="129" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="F32" s="58" t="n"/>
+      <c r="G32" s="58" t="n"/>
+      <c r="H32" s="129" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="I32" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J32" s="129" t="inlineStr"/>
+    </row>
+    <row r="33" ht="16" customHeight="1" s="28">
+      <c r="A33" s="129" t="n">
+        <v>24</v>
+      </c>
+      <c r="B33" s="129" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C33" s="129" t="inlineStr">
+        <is>
+          <t>Group D</t>
+        </is>
+      </c>
+      <c r="D33" s="129" t="inlineStr"/>
+      <c r="E33" s="129" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="F33" s="58" t="n"/>
+      <c r="G33" s="58" t="n"/>
+      <c r="H33" s="129" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="I33" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J33" s="129" t="inlineStr"/>
+    </row>
+    <row r="34"/>
+    <row r="35" ht="18" customHeight="1" s="28">
+      <c r="A35" s="130" t="inlineStr">
+        <is>
+          <t>Group E  –  Germany | Ecuador | Ivory Coast | Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="16" customHeight="1" s="28">
+      <c r="A36" s="131" t="n">
+        <v>25</v>
+      </c>
+      <c r="B36" s="131" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C36" s="131" t="inlineStr">
+        <is>
+          <t>Group E</t>
+        </is>
+      </c>
+      <c r="D36" s="131" t="inlineStr"/>
+      <c r="E36" s="131" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F36" s="58" t="n"/>
+      <c r="G36" s="58" t="n"/>
+      <c r="H36" s="131" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="I36" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J36" s="131" t="inlineStr"/>
+    </row>
+    <row r="37" ht="16" customHeight="1" s="28">
+      <c r="A37" s="131" t="n">
+        <v>26</v>
+      </c>
+      <c r="B37" s="131" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C37" s="131" t="inlineStr">
+        <is>
+          <t>Group E</t>
+        </is>
+      </c>
+      <c r="D37" s="131" t="inlineStr"/>
+      <c r="E37" s="131" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F37" s="58" t="n"/>
+      <c r="G37" s="58" t="n"/>
+      <c r="H37" s="131" t="inlineStr">
+        <is>
+          <t>Ivory Coast</t>
+        </is>
+      </c>
+      <c r="I37" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J37" s="131" t="inlineStr"/>
+    </row>
+    <row r="38" ht="16" customHeight="1" s="28">
+      <c r="A38" s="131" t="n">
+        <v>27</v>
+      </c>
+      <c r="B38" s="131" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C38" s="131" t="inlineStr">
+        <is>
+          <t>Group E</t>
+        </is>
+      </c>
+      <c r="D38" s="131" t="inlineStr"/>
+      <c r="E38" s="131" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F38" s="58" t="n"/>
+      <c r="G38" s="58" t="n"/>
+      <c r="H38" s="131" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+      <c r="I38" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J38" s="131" t="inlineStr"/>
+    </row>
+    <row r="39" ht="16" customHeight="1" s="28">
+      <c r="A39" s="131" t="n">
+        <v>28</v>
+      </c>
+      <c r="B39" s="131" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C39" s="131" t="inlineStr">
+        <is>
+          <t>Group E</t>
+        </is>
+      </c>
+      <c r="D39" s="131" t="inlineStr"/>
+      <c r="E39" s="131" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="F39" s="58" t="n"/>
+      <c r="G39" s="58" t="n"/>
+      <c r="H39" s="131" t="inlineStr">
+        <is>
+          <t>Ivory Coast</t>
+        </is>
+      </c>
+      <c r="I39" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J39" s="131" t="inlineStr"/>
+    </row>
+    <row r="40" ht="16" customHeight="1" s="28">
+      <c r="A40" s="131" t="n">
+        <v>29</v>
+      </c>
+      <c r="B40" s="131" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C40" s="131" t="inlineStr">
+        <is>
+          <t>Group E</t>
+        </is>
+      </c>
+      <c r="D40" s="131" t="inlineStr"/>
+      <c r="E40" s="131" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="F40" s="58" t="n"/>
+      <c r="G40" s="58" t="n"/>
+      <c r="H40" s="131" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+      <c r="I40" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J40" s="131" t="inlineStr"/>
+    </row>
+    <row r="41" ht="16" customHeight="1" s="28">
+      <c r="A41" s="131" t="n">
+        <v>30</v>
+      </c>
+      <c r="B41" s="131" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C41" s="131" t="inlineStr">
+        <is>
+          <t>Group E</t>
+        </is>
+      </c>
+      <c r="D41" s="131" t="inlineStr"/>
+      <c r="E41" s="131" t="inlineStr">
+        <is>
+          <t>Ivory Coast</t>
+        </is>
+      </c>
+      <c r="F41" s="58" t="n"/>
+      <c r="G41" s="58" t="n"/>
+      <c r="H41" s="131" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+      <c r="I41" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J41" s="131" t="inlineStr"/>
+    </row>
+    <row r="42"/>
+    <row r="43" ht="18" customHeight="1" s="28">
+      <c r="A43" s="132" t="inlineStr">
+        <is>
+          <t>Group F  –  Netherlands | Japan | Sweden | Tunisia</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="16" customHeight="1" s="28">
+      <c r="A44" s="133" t="n">
+        <v>31</v>
+      </c>
+      <c r="B44" s="133" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C44" s="133" t="inlineStr">
+        <is>
+          <t>Group F</t>
+        </is>
+      </c>
+      <c r="D44" s="133" t="inlineStr"/>
+      <c r="E44" s="133" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="F44" s="58" t="n"/>
+      <c r="G44" s="58" t="n"/>
+      <c r="H44" s="133" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="I44" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J44" s="133" t="inlineStr"/>
+    </row>
+    <row r="45" ht="16" customHeight="1" s="28">
+      <c r="A45" s="133" t="n">
+        <v>32</v>
+      </c>
+      <c r="B45" s="133" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C45" s="133" t="inlineStr">
+        <is>
+          <t>Group F</t>
+        </is>
+      </c>
+      <c r="D45" s="133" t="inlineStr"/>
+      <c r="E45" s="133" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="F45" s="58" t="n"/>
+      <c r="G45" s="58" t="n"/>
+      <c r="H45" s="133" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="I45" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J45" s="133" t="inlineStr"/>
+    </row>
+    <row r="46" ht="16" customHeight="1" s="28">
+      <c r="A46" s="133" t="n">
+        <v>33</v>
+      </c>
+      <c r="B46" s="133" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C46" s="133" t="inlineStr">
+        <is>
+          <t>Group F</t>
+        </is>
+      </c>
+      <c r="D46" s="133" t="inlineStr"/>
+      <c r="E46" s="133" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="F46" s="58" t="n"/>
+      <c r="G46" s="58" t="n"/>
+      <c r="H46" s="133" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="I46" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J46" s="133" t="inlineStr"/>
+    </row>
+    <row r="47" ht="16" customHeight="1" s="28">
+      <c r="A47" s="133" t="n">
+        <v>34</v>
+      </c>
+      <c r="B47" s="133" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C47" s="133" t="inlineStr">
+        <is>
+          <t>Group F</t>
+        </is>
+      </c>
+      <c r="D47" s="133" t="inlineStr"/>
+      <c r="E47" s="133" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F47" s="58" t="n"/>
+      <c r="G47" s="58" t="n"/>
+      <c r="H47" s="133" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="I47" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J47" s="133" t="inlineStr"/>
+    </row>
+    <row r="48" ht="16" customHeight="1" s="28">
+      <c r="A48" s="133" t="n">
+        <v>35</v>
+      </c>
+      <c r="B48" s="133" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C48" s="133" t="inlineStr">
+        <is>
+          <t>Group F</t>
+        </is>
+      </c>
+      <c r="D48" s="133" t="inlineStr"/>
+      <c r="E48" s="133" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F48" s="58" t="n"/>
+      <c r="G48" s="58" t="n"/>
+      <c r="H48" s="133" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="I48" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J48" s="133" t="inlineStr"/>
+    </row>
+    <row r="49" ht="16" customHeight="1" s="28">
+      <c r="A49" s="133" t="n">
+        <v>36</v>
+      </c>
+      <c r="B49" s="133" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C49" s="133" t="inlineStr">
+        <is>
+          <t>Group F</t>
+        </is>
+      </c>
+      <c r="D49" s="133" t="inlineStr"/>
+      <c r="E49" s="133" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F49" s="58" t="n"/>
+      <c r="G49" s="58" t="n"/>
+      <c r="H49" s="133" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="I49" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J49" s="133" t="inlineStr"/>
+    </row>
+    <row r="50"/>
+    <row r="51" ht="18" customHeight="1" s="28">
+      <c r="A51" s="134" t="inlineStr">
+        <is>
+          <t>Group G  –  Belgium | Egypt | Iran | New Zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="16" customHeight="1" s="28">
+      <c r="A52" s="135" t="n">
+        <v>37</v>
+      </c>
+      <c r="B52" s="135" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C52" s="135" t="inlineStr">
+        <is>
+          <t>Group G</t>
+        </is>
+      </c>
+      <c r="D52" s="135" t="inlineStr"/>
+      <c r="E52" s="135" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="F52" s="58" t="n"/>
+      <c r="G52" s="58" t="n"/>
+      <c r="H52" s="135" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="I52" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J52" s="135" t="inlineStr"/>
+    </row>
+    <row r="53" ht="16" customHeight="1" s="28">
+      <c r="A53" s="135" t="n">
+        <v>38</v>
+      </c>
+      <c r="B53" s="135" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C53" s="135" t="inlineStr">
+        <is>
+          <t>Group G</t>
+        </is>
+      </c>
+      <c r="D53" s="135" t="inlineStr"/>
+      <c r="E53" s="135" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="F53" s="58" t="n"/>
+      <c r="G53" s="58" t="n"/>
+      <c r="H53" s="135" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="I53" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J53" s="135" t="inlineStr"/>
+    </row>
+    <row r="54" ht="16" customHeight="1" s="28">
+      <c r="A54" s="135" t="n">
+        <v>39</v>
+      </c>
+      <c r="B54" s="135" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C54" s="135" t="inlineStr">
+        <is>
+          <t>Group G</t>
+        </is>
+      </c>
+      <c r="D54" s="135" t="inlineStr"/>
+      <c r="E54" s="135" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="F54" s="58" t="n"/>
+      <c r="G54" s="58" t="n"/>
+      <c r="H54" s="135" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="I54" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J54" s="135" t="inlineStr"/>
+    </row>
+    <row r="55" ht="16" customHeight="1" s="28">
+      <c r="A55" s="135" t="n">
+        <v>40</v>
+      </c>
+      <c r="B55" s="135" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C55" s="135" t="inlineStr">
+        <is>
+          <t>Group G</t>
+        </is>
+      </c>
+      <c r="D55" s="135" t="inlineStr"/>
+      <c r="E55" s="135" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="F55" s="58" t="n"/>
+      <c r="G55" s="58" t="n"/>
+      <c r="H55" s="135" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="I55" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J55" s="135" t="inlineStr"/>
+    </row>
+    <row r="56" ht="16" customHeight="1" s="28">
+      <c r="A56" s="135" t="n">
+        <v>41</v>
+      </c>
+      <c r="B56" s="135" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C56" s="135" t="inlineStr">
+        <is>
+          <t>Group G</t>
+        </is>
+      </c>
+      <c r="D56" s="135" t="inlineStr"/>
+      <c r="E56" s="135" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="F56" s="58" t="n"/>
+      <c r="G56" s="58" t="n"/>
+      <c r="H56" s="135" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="I56" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J56" s="135" t="inlineStr"/>
+    </row>
+    <row r="57" ht="16" customHeight="1" s="28">
+      <c r="A57" s="135" t="n">
+        <v>42</v>
+      </c>
+      <c r="B57" s="135" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C57" s="135" t="inlineStr">
+        <is>
+          <t>Group G</t>
+        </is>
+      </c>
+      <c r="D57" s="135" t="inlineStr"/>
+      <c r="E57" s="135" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="F57" s="58" t="n"/>
+      <c r="G57" s="58" t="n"/>
+      <c r="H57" s="135" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="I57" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J57" s="135" t="inlineStr"/>
+    </row>
+    <row r="58"/>
+    <row r="59" ht="18" customHeight="1" s="28">
+      <c r="A59" s="136" t="inlineStr">
+        <is>
+          <t>Group H  –  Spain | Uruguay | Saudi Arabia | Cape Verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="16" customHeight="1" s="28">
+      <c r="A60" s="137" t="n">
+        <v>43</v>
+      </c>
+      <c r="B60" s="137" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C60" s="137" t="inlineStr">
+        <is>
+          <t>Group H</t>
+        </is>
+      </c>
+      <c r="D60" s="137" t="inlineStr"/>
+      <c r="E60" s="137" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="F60" s="58" t="n"/>
+      <c r="G60" s="58" t="n"/>
+      <c r="H60" s="137" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="I60" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J60" s="137" t="inlineStr"/>
+    </row>
+    <row r="61" ht="16" customHeight="1" s="28">
+      <c r="A61" s="137" t="n">
+        <v>44</v>
+      </c>
+      <c r="B61" s="137" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C61" s="137" t="inlineStr">
+        <is>
+          <t>Group H</t>
+        </is>
+      </c>
+      <c r="D61" s="137" t="inlineStr"/>
+      <c r="E61" s="137" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="F61" s="58" t="n"/>
+      <c r="G61" s="58" t="n"/>
+      <c r="H61" s="137" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="I61" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J61" s="137" t="inlineStr"/>
+    </row>
+    <row r="62" ht="16" customHeight="1" s="28">
+      <c r="A62" s="137" t="n">
+        <v>45</v>
+      </c>
+      <c r="B62" s="137" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C62" s="137" t="inlineStr">
+        <is>
+          <t>Group H</t>
+        </is>
+      </c>
+      <c r="D62" s="137" t="inlineStr"/>
+      <c r="E62" s="137" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="F62" s="58" t="n"/>
+      <c r="G62" s="58" t="n"/>
+      <c r="H62" s="137" t="inlineStr">
+        <is>
+          <t>Cape Verde</t>
+        </is>
+      </c>
+      <c r="I62" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J62" s="137" t="inlineStr"/>
+    </row>
+    <row r="63" ht="16" customHeight="1" s="28">
+      <c r="A63" s="137" t="n">
+        <v>46</v>
+      </c>
+      <c r="B63" s="137" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C63" s="137" t="inlineStr">
+        <is>
+          <t>Group H</t>
+        </is>
+      </c>
+      <c r="D63" s="137" t="inlineStr"/>
+      <c r="E63" s="137" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="F63" s="58" t="n"/>
+      <c r="G63" s="58" t="n"/>
+      <c r="H63" s="137" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="I63" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J63" s="137" t="inlineStr"/>
+    </row>
+    <row r="64" ht="16" customHeight="1" s="28">
+      <c r="A64" s="137" t="n">
+        <v>47</v>
+      </c>
+      <c r="B64" s="137" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C64" s="137" t="inlineStr">
+        <is>
+          <t>Group H</t>
+        </is>
+      </c>
+      <c r="D64" s="137" t="inlineStr"/>
+      <c r="E64" s="137" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="F64" s="58" t="n"/>
+      <c r="G64" s="58" t="n"/>
+      <c r="H64" s="137" t="inlineStr">
+        <is>
+          <t>Cape Verde</t>
+        </is>
+      </c>
+      <c r="I64" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J64" s="137" t="inlineStr"/>
+    </row>
+    <row r="65" ht="16" customHeight="1" s="28">
+      <c r="A65" s="137" t="n">
+        <v>48</v>
+      </c>
+      <c r="B65" s="137" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C65" s="137" t="inlineStr">
+        <is>
+          <t>Group H</t>
+        </is>
+      </c>
+      <c r="D65" s="137" t="inlineStr"/>
+      <c r="E65" s="137" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="F65" s="58" t="n"/>
+      <c r="G65" s="58" t="n"/>
+      <c r="H65" s="137" t="inlineStr">
+        <is>
+          <t>Cape Verde</t>
+        </is>
+      </c>
+      <c r="I65" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J65" s="137" t="inlineStr"/>
+    </row>
+    <row r="66"/>
+    <row r="67" ht="18" customHeight="1" s="28">
+      <c r="A67" s="138" t="inlineStr">
+        <is>
+          <t>Group I  –  France | Senegal | Norway | Iraq</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="16" customHeight="1" s="28">
+      <c r="A68" s="139" t="n">
+        <v>49</v>
+      </c>
+      <c r="B68" s="139" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C68" s="139" t="inlineStr">
+        <is>
+          <t>Group I</t>
+        </is>
+      </c>
+      <c r="D68" s="139" t="inlineStr"/>
+      <c r="E68" s="139" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="F68" s="58" t="n"/>
+      <c r="G68" s="58" t="n"/>
+      <c r="H68" s="139" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="I68" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J68" s="139" t="inlineStr"/>
+    </row>
+    <row r="69" ht="16" customHeight="1" s="28">
+      <c r="A69" s="139" t="n">
+        <v>50</v>
+      </c>
+      <c r="B69" s="139" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C69" s="139" t="inlineStr">
+        <is>
+          <t>Group I</t>
+        </is>
+      </c>
+      <c r="D69" s="139" t="inlineStr"/>
+      <c r="E69" s="139" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="F69" s="58" t="n"/>
+      <c r="G69" s="58" t="n"/>
+      <c r="H69" s="139" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="I69" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J69" s="139" t="inlineStr"/>
+    </row>
+    <row r="70" ht="16" customHeight="1" s="28">
+      <c r="A70" s="139" t="n">
+        <v>51</v>
+      </c>
+      <c r="B70" s="139" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C70" s="139" t="inlineStr">
+        <is>
+          <t>Group I</t>
+        </is>
+      </c>
+      <c r="D70" s="139" t="inlineStr"/>
+      <c r="E70" s="139" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="F70" s="58" t="n"/>
+      <c r="G70" s="58" t="n"/>
+      <c r="H70" s="139" t="inlineStr">
+        <is>
+          <t>Iraq</t>
+        </is>
+      </c>
+      <c r="I70" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J70" s="139" t="inlineStr"/>
+    </row>
+    <row r="71" ht="16" customHeight="1" s="28">
+      <c r="A71" s="139" t="n">
+        <v>52</v>
+      </c>
+      <c r="B71" s="139" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C71" s="139" t="inlineStr">
+        <is>
+          <t>Group I</t>
+        </is>
+      </c>
+      <c r="D71" s="139" t="inlineStr"/>
+      <c r="E71" s="139" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="F71" s="58" t="n"/>
+      <c r="G71" s="58" t="n"/>
+      <c r="H71" s="139" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="I71" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J71" s="139" t="inlineStr"/>
+    </row>
+    <row r="72" ht="16" customHeight="1" s="28">
+      <c r="A72" s="139" t="n">
+        <v>53</v>
+      </c>
+      <c r="B72" s="139" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C72" s="139" t="inlineStr">
+        <is>
+          <t>Group I</t>
+        </is>
+      </c>
+      <c r="D72" s="139" t="inlineStr"/>
+      <c r="E72" s="139" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="F72" s="58" t="n"/>
+      <c r="G72" s="58" t="n"/>
+      <c r="H72" s="139" t="inlineStr">
+        <is>
+          <t>Iraq</t>
+        </is>
+      </c>
+      <c r="I72" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J72" s="139" t="inlineStr"/>
+    </row>
+    <row r="73" ht="16" customHeight="1" s="28">
+      <c r="A73" s="139" t="n">
+        <v>54</v>
+      </c>
+      <c r="B73" s="139" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C73" s="139" t="inlineStr">
+        <is>
+          <t>Group I</t>
+        </is>
+      </c>
+      <c r="D73" s="139" t="inlineStr"/>
+      <c r="E73" s="139" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="F73" s="58" t="n"/>
+      <c r="G73" s="58" t="n"/>
+      <c r="H73" s="139" t="inlineStr">
+        <is>
+          <t>Iraq</t>
+        </is>
+      </c>
+      <c r="I73" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J73" s="139" t="inlineStr"/>
+    </row>
+    <row r="74"/>
+    <row r="75" ht="18" customHeight="1" s="28">
+      <c r="A75" s="140" t="inlineStr">
+        <is>
+          <t>Group J  –  Argentina | Austria | Algeria | Jordan</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="16" customHeight="1" s="28">
+      <c r="A76" s="141" t="n">
+        <v>55</v>
+      </c>
+      <c r="B76" s="141" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C76" s="141" t="inlineStr">
+        <is>
+          <t>Group J</t>
+        </is>
+      </c>
+      <c r="D76" s="141" t="inlineStr"/>
+      <c r="E76" s="141" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F76" s="58" t="n"/>
+      <c r="G76" s="58" t="n"/>
+      <c r="H76" s="141" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="I76" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J76" s="141" t="inlineStr"/>
+    </row>
+    <row r="77" ht="16" customHeight="1" s="28">
+      <c r="A77" s="141" t="n">
+        <v>56</v>
+      </c>
+      <c r="B77" s="141" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C77" s="141" t="inlineStr">
+        <is>
+          <t>Group J</t>
+        </is>
+      </c>
+      <c r="D77" s="141" t="inlineStr"/>
+      <c r="E77" s="141" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F77" s="58" t="n"/>
+      <c r="G77" s="58" t="n"/>
+      <c r="H77" s="141" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="I77" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J77" s="141" t="inlineStr"/>
+    </row>
+    <row r="78" ht="16" customHeight="1" s="28">
+      <c r="A78" s="141" t="n">
+        <v>57</v>
+      </c>
+      <c r="B78" s="141" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C78" s="141" t="inlineStr">
+        <is>
+          <t>Group J</t>
+        </is>
+      </c>
+      <c r="D78" s="141" t="inlineStr"/>
+      <c r="E78" s="141" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F78" s="58" t="n"/>
+      <c r="G78" s="58" t="n"/>
+      <c r="H78" s="141" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="I78" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J78" s="141" t="inlineStr"/>
+    </row>
+    <row r="79" ht="16" customHeight="1" s="28">
+      <c r="A79" s="141" t="n">
+        <v>58</v>
+      </c>
+      <c r="B79" s="141" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C79" s="141" t="inlineStr">
+        <is>
+          <t>Group J</t>
+        </is>
+      </c>
+      <c r="D79" s="141" t="inlineStr"/>
+      <c r="E79" s="141" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="F79" s="58" t="n"/>
+      <c r="G79" s="58" t="n"/>
+      <c r="H79" s="141" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="I79" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J79" s="141" t="inlineStr"/>
+    </row>
+    <row r="80" ht="16" customHeight="1" s="28">
+      <c r="A80" s="141" t="n">
+        <v>59</v>
+      </c>
+      <c r="B80" s="141" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C80" s="141" t="inlineStr">
+        <is>
+          <t>Group J</t>
+        </is>
+      </c>
+      <c r="D80" s="141" t="inlineStr"/>
+      <c r="E80" s="141" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="F80" s="58" t="n"/>
+      <c r="G80" s="58" t="n"/>
+      <c r="H80" s="141" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="I80" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J80" s="141" t="inlineStr"/>
+    </row>
+    <row r="81" ht="16" customHeight="1" s="28">
+      <c r="A81" s="141" t="n">
+        <v>60</v>
+      </c>
+      <c r="B81" s="141" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C81" s="141" t="inlineStr">
+        <is>
+          <t>Group J</t>
+        </is>
+      </c>
+      <c r="D81" s="141" t="inlineStr"/>
+      <c r="E81" s="141" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="F81" s="58" t="n"/>
+      <c r="G81" s="58" t="n"/>
+      <c r="H81" s="141" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="I81" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J81" s="141" t="inlineStr"/>
+    </row>
+    <row r="82"/>
+    <row r="83" ht="18" customHeight="1" s="28">
+      <c r="A83" s="130" t="inlineStr">
+        <is>
+          <t>Group K  –  Portugal | Colombia | Uzbekistan | DR Congo</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="16" customHeight="1" s="28">
+      <c r="A84" s="131" t="n">
+        <v>61</v>
+      </c>
+      <c r="B84" s="131" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C84" s="131" t="inlineStr">
+        <is>
+          <t>Group K</t>
+        </is>
+      </c>
+      <c r="D84" s="131" t="inlineStr"/>
+      <c r="E84" s="131" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="F84" s="58" t="n"/>
+      <c r="G84" s="58" t="n"/>
+      <c r="H84" s="131" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="I84" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J84" s="131" t="inlineStr"/>
+    </row>
+    <row r="85" ht="16" customHeight="1" s="28">
+      <c r="A85" s="131" t="n">
+        <v>62</v>
+      </c>
+      <c r="B85" s="131" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C85" s="131" t="inlineStr">
+        <is>
+          <t>Group K</t>
+        </is>
+      </c>
+      <c r="D85" s="131" t="inlineStr"/>
+      <c r="E85" s="131" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="F85" s="58" t="n"/>
+      <c r="G85" s="58" t="n"/>
+      <c r="H85" s="131" t="inlineStr">
+        <is>
+          <t>Uzbekistan</t>
+        </is>
+      </c>
+      <c r="I85" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J85" s="131" t="inlineStr"/>
+    </row>
+    <row r="86" ht="16" customHeight="1" s="28">
+      <c r="A86" s="131" t="n">
+        <v>63</v>
+      </c>
+      <c r="B86" s="131" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C86" s="131" t="inlineStr">
+        <is>
+          <t>Group K</t>
+        </is>
+      </c>
+      <c r="D86" s="131" t="inlineStr"/>
+      <c r="E86" s="131" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="F86" s="58" t="n"/>
+      <c r="G86" s="58" t="n"/>
+      <c r="H86" s="131" t="inlineStr">
+        <is>
+          <t>DR Congo</t>
+        </is>
+      </c>
+      <c r="I86" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J86" s="131" t="inlineStr"/>
+    </row>
+    <row r="87" ht="16" customHeight="1" s="28">
+      <c r="A87" s="131" t="n">
+        <v>64</v>
+      </c>
+      <c r="B87" s="131" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C87" s="131" t="inlineStr">
+        <is>
+          <t>Group K</t>
+        </is>
+      </c>
+      <c r="D87" s="131" t="inlineStr"/>
+      <c r="E87" s="131" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="F87" s="58" t="n"/>
+      <c r="G87" s="58" t="n"/>
+      <c r="H87" s="131" t="inlineStr">
+        <is>
+          <t>Uzbekistan</t>
+        </is>
+      </c>
+      <c r="I87" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J87" s="131" t="inlineStr"/>
+    </row>
+    <row r="88" ht="16" customHeight="1" s="28">
+      <c r="A88" s="131" t="n">
+        <v>65</v>
+      </c>
+      <c r="B88" s="131" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C88" s="131" t="inlineStr">
+        <is>
+          <t>Group K</t>
+        </is>
+      </c>
+      <c r="D88" s="131" t="inlineStr"/>
+      <c r="E88" s="131" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="F88" s="58" t="n"/>
+      <c r="G88" s="58" t="n"/>
+      <c r="H88" s="131" t="inlineStr">
+        <is>
+          <t>DR Congo</t>
+        </is>
+      </c>
+      <c r="I88" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J88" s="131" t="inlineStr"/>
+    </row>
+    <row r="89" ht="16" customHeight="1" s="28">
+      <c r="A89" s="131" t="n">
+        <v>66</v>
+      </c>
+      <c r="B89" s="131" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C89" s="131" t="inlineStr">
+        <is>
+          <t>Group K</t>
+        </is>
+      </c>
+      <c r="D89" s="131" t="inlineStr"/>
+      <c r="E89" s="131" t="inlineStr">
+        <is>
+          <t>Uzbekistan</t>
+        </is>
+      </c>
+      <c r="F89" s="58" t="n"/>
+      <c r="G89" s="58" t="n"/>
+      <c r="H89" s="131" t="inlineStr">
+        <is>
+          <t>DR Congo</t>
+        </is>
+      </c>
+      <c r="I89" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J89" s="131" t="inlineStr"/>
+    </row>
+    <row r="90"/>
+    <row r="91" ht="18" customHeight="1" s="28">
+      <c r="A91" s="142" t="inlineStr">
+        <is>
+          <t>Group L  –  England | Croatia | Ghana | Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="16" customHeight="1" s="28">
+      <c r="A92" s="143" t="n">
+        <v>67</v>
+      </c>
+      <c r="B92" s="143" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C92" s="143" t="inlineStr">
+        <is>
+          <t>Group L</t>
+        </is>
+      </c>
+      <c r="D92" s="143" t="inlineStr"/>
+      <c r="E92" s="143" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F92" s="58" t="n"/>
+      <c r="G92" s="58" t="n"/>
+      <c r="H92" s="143" t="inlineStr">
+        <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="I92" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J92" s="143" t="inlineStr"/>
+    </row>
+    <row r="93" ht="16" customHeight="1" s="28">
+      <c r="A93" s="143" t="n">
+        <v>68</v>
+      </c>
+      <c r="B93" s="143" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C93" s="143" t="inlineStr">
+        <is>
+          <t>Group L</t>
+        </is>
+      </c>
+      <c r="D93" s="143" t="inlineStr"/>
+      <c r="E93" s="143" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F93" s="58" t="n"/>
+      <c r="G93" s="58" t="n"/>
+      <c r="H93" s="143" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="I93" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J93" s="143" t="inlineStr"/>
+    </row>
+    <row r="94" ht="16" customHeight="1" s="28">
+      <c r="A94" s="143" t="n">
+        <v>69</v>
+      </c>
+      <c r="B94" s="143" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C94" s="143" t="inlineStr">
+        <is>
+          <t>Group L</t>
+        </is>
+      </c>
+      <c r="D94" s="143" t="inlineStr"/>
+      <c r="E94" s="143" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F94" s="58" t="n"/>
+      <c r="G94" s="58" t="n"/>
+      <c r="H94" s="143" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="I94" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J94" s="143" t="inlineStr"/>
+    </row>
+    <row r="95" ht="16" customHeight="1" s="28">
+      <c r="A95" s="143" t="n">
+        <v>70</v>
+      </c>
+      <c r="B95" s="143" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C95" s="143" t="inlineStr">
+        <is>
+          <t>Group L</t>
+        </is>
+      </c>
+      <c r="D95" s="143" t="inlineStr"/>
+      <c r="E95" s="143" t="inlineStr">
+        <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="F95" s="58" t="n"/>
+      <c r="G95" s="58" t="n"/>
+      <c r="H95" s="143" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="I95" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J95" s="143" t="inlineStr"/>
+    </row>
+    <row r="96" ht="16" customHeight="1" s="28">
+      <c r="A96" s="143" t="n">
+        <v>71</v>
+      </c>
+      <c r="B96" s="143" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C96" s="143" t="inlineStr">
+        <is>
+          <t>Group L</t>
+        </is>
+      </c>
+      <c r="D96" s="143" t="inlineStr"/>
+      <c r="E96" s="143" t="inlineStr">
+        <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="F96" s="58" t="n"/>
+      <c r="G96" s="58" t="n"/>
+      <c r="H96" s="143" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="I96" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J96" s="143" t="inlineStr"/>
+    </row>
+    <row r="97" ht="16" customHeight="1" s="28">
+      <c r="A97" s="143" t="n">
+        <v>72</v>
+      </c>
+      <c r="B97" s="143" t="inlineStr">
+        <is>
+          <t>Group Stage</t>
+        </is>
+      </c>
+      <c r="C97" s="143" t="inlineStr">
+        <is>
+          <t>Group L</t>
+        </is>
+      </c>
+      <c r="D97" s="143" t="inlineStr"/>
+      <c r="E97" s="143" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="F97" s="58" t="n"/>
+      <c r="G97" s="58" t="n"/>
+      <c r="H97" s="143" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="I97" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J97" s="143" t="inlineStr"/>
+    </row>
+    <row r="98"/>
+    <row r="99" ht="22" customHeight="1" s="28">
+      <c r="A99" s="144" t="inlineStr">
+        <is>
+          <t>KNOCKOUT ROUNDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="18" customHeight="1" s="28">
+      <c r="A100" s="145" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="16" customHeight="1" s="28">
+      <c r="A101" s="60" t="n">
+        <v>73</v>
+      </c>
+      <c r="B101" s="60" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C101" s="60" t="inlineStr"/>
+      <c r="D101" s="60" t="inlineStr"/>
+      <c r="E101" s="60" t="inlineStr"/>
+      <c r="F101" s="58" t="n"/>
+      <c r="G101" s="58" t="n"/>
+      <c r="H101" s="60" t="inlineStr"/>
+      <c r="I101" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J101" s="60" t="inlineStr"/>
+    </row>
+    <row r="102" ht="16" customHeight="1" s="28">
+      <c r="A102" s="57" t="n">
+        <v>74</v>
+      </c>
+      <c r="B102" s="57" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C102" s="57" t="inlineStr"/>
+      <c r="D102" s="57" t="inlineStr"/>
+      <c r="E102" s="57" t="inlineStr"/>
+      <c r="F102" s="58" t="n"/>
+      <c r="G102" s="58" t="n"/>
+      <c r="H102" s="57" t="inlineStr"/>
+      <c r="I102" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J102" s="57" t="inlineStr"/>
+    </row>
+    <row r="103" ht="16" customHeight="1" s="28">
+      <c r="A103" s="60" t="n">
+        <v>75</v>
+      </c>
+      <c r="B103" s="60" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C103" s="60" t="inlineStr"/>
+      <c r="D103" s="60" t="inlineStr"/>
+      <c r="E103" s="60" t="inlineStr"/>
+      <c r="F103" s="58" t="n"/>
+      <c r="G103" s="58" t="n"/>
+      <c r="H103" s="60" t="inlineStr"/>
+      <c r="I103" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J103" s="60" t="inlineStr"/>
+    </row>
+    <row r="104" ht="16" customHeight="1" s="28">
+      <c r="A104" s="57" t="n">
+        <v>76</v>
+      </c>
+      <c r="B104" s="57" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C104" s="57" t="inlineStr"/>
+      <c r="D104" s="57" t="inlineStr"/>
+      <c r="E104" s="57" t="inlineStr"/>
+      <c r="F104" s="58" t="n"/>
+      <c r="G104" s="58" t="n"/>
+      <c r="H104" s="57" t="inlineStr"/>
+      <c r="I104" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J104" s="57" t="inlineStr"/>
+    </row>
+    <row r="105" ht="16" customHeight="1" s="28">
+      <c r="A105" s="60" t="n">
+        <v>77</v>
+      </c>
+      <c r="B105" s="60" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C105" s="60" t="inlineStr"/>
+      <c r="D105" s="60" t="inlineStr"/>
+      <c r="E105" s="60" t="inlineStr"/>
+      <c r="F105" s="58" t="n"/>
+      <c r="G105" s="58" t="n"/>
+      <c r="H105" s="60" t="inlineStr"/>
+      <c r="I105" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J105" s="60" t="inlineStr"/>
+    </row>
+    <row r="106" ht="16" customHeight="1" s="28">
+      <c r="A106" s="57" t="n">
+        <v>78</v>
+      </c>
+      <c r="B106" s="57" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C106" s="57" t="inlineStr"/>
+      <c r="D106" s="57" t="inlineStr"/>
+      <c r="E106" s="57" t="inlineStr"/>
+      <c r="F106" s="58" t="n"/>
+      <c r="G106" s="58" t="n"/>
+      <c r="H106" s="57" t="inlineStr"/>
+      <c r="I106" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J106" s="57" t="inlineStr"/>
+    </row>
+    <row r="107" ht="16" customHeight="1" s="28">
+      <c r="A107" s="60" t="n">
+        <v>79</v>
+      </c>
+      <c r="B107" s="60" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C107" s="60" t="inlineStr"/>
+      <c r="D107" s="60" t="inlineStr"/>
+      <c r="E107" s="60" t="inlineStr"/>
+      <c r="F107" s="58" t="n"/>
+      <c r="G107" s="58" t="n"/>
+      <c r="H107" s="60" t="inlineStr"/>
+      <c r="I107" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J107" s="60" t="inlineStr"/>
+    </row>
+    <row r="108" ht="16" customHeight="1" s="28">
+      <c r="A108" s="57" t="n">
+        <v>80</v>
+      </c>
+      <c r="B108" s="57" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C108" s="57" t="inlineStr"/>
+      <c r="D108" s="57" t="inlineStr"/>
+      <c r="E108" s="57" t="inlineStr"/>
+      <c r="F108" s="58" t="n"/>
+      <c r="G108" s="58" t="n"/>
+      <c r="H108" s="57" t="inlineStr"/>
+      <c r="I108" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J108" s="57" t="inlineStr"/>
+    </row>
+    <row r="109" ht="16" customHeight="1" s="28">
+      <c r="A109" s="60" t="n">
+        <v>81</v>
+      </c>
+      <c r="B109" s="60" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C109" s="60" t="inlineStr"/>
+      <c r="D109" s="60" t="inlineStr"/>
+      <c r="E109" s="60" t="inlineStr"/>
+      <c r="F109" s="58" t="n"/>
+      <c r="G109" s="58" t="n"/>
+      <c r="H109" s="60" t="inlineStr"/>
+      <c r="I109" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J109" s="60" t="inlineStr"/>
+    </row>
+    <row r="110" ht="16" customHeight="1" s="28">
+      <c r="A110" s="57" t="n">
+        <v>82</v>
+      </c>
+      <c r="B110" s="57" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C110" s="57" t="inlineStr"/>
+      <c r="D110" s="57" t="inlineStr"/>
+      <c r="E110" s="57" t="inlineStr"/>
+      <c r="F110" s="58" t="n"/>
+      <c r="G110" s="58" t="n"/>
+      <c r="H110" s="57" t="inlineStr"/>
+      <c r="I110" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J110" s="57" t="inlineStr"/>
+    </row>
+    <row r="111" ht="16" customHeight="1" s="28">
+      <c r="A111" s="60" t="n">
+        <v>83</v>
+      </c>
+      <c r="B111" s="60" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C111" s="60" t="inlineStr"/>
+      <c r="D111" s="60" t="inlineStr"/>
+      <c r="E111" s="60" t="inlineStr"/>
+      <c r="F111" s="58" t="n"/>
+      <c r="G111" s="58" t="n"/>
+      <c r="H111" s="60" t="inlineStr"/>
+      <c r="I111" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J111" s="60" t="inlineStr"/>
+    </row>
+    <row r="112" ht="16" customHeight="1" s="28">
+      <c r="A112" s="57" t="n">
+        <v>84</v>
+      </c>
+      <c r="B112" s="57" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C112" s="57" t="inlineStr"/>
+      <c r="D112" s="57" t="inlineStr"/>
+      <c r="E112" s="57" t="inlineStr"/>
+      <c r="F112" s="58" t="n"/>
+      <c r="G112" s="58" t="n"/>
+      <c r="H112" s="57" t="inlineStr"/>
+      <c r="I112" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J112" s="57" t="inlineStr"/>
+    </row>
+    <row r="113" ht="16" customHeight="1" s="28">
+      <c r="A113" s="60" t="n">
+        <v>85</v>
+      </c>
+      <c r="B113" s="60" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C113" s="60" t="inlineStr"/>
+      <c r="D113" s="60" t="inlineStr"/>
+      <c r="E113" s="60" t="inlineStr"/>
+      <c r="F113" s="58" t="n"/>
+      <c r="G113" s="58" t="n"/>
+      <c r="H113" s="60" t="inlineStr"/>
+      <c r="I113" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J113" s="60" t="inlineStr"/>
+    </row>
+    <row r="114" ht="16" customHeight="1" s="28">
+      <c r="A114" s="57" t="n">
+        <v>86</v>
+      </c>
+      <c r="B114" s="57" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C114" s="57" t="inlineStr"/>
+      <c r="D114" s="57" t="inlineStr"/>
+      <c r="E114" s="57" t="inlineStr"/>
+      <c r="F114" s="58" t="n"/>
+      <c r="G114" s="58" t="n"/>
+      <c r="H114" s="57" t="inlineStr"/>
+      <c r="I114" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J114" s="57" t="inlineStr"/>
+    </row>
+    <row r="115" ht="16" customHeight="1" s="28">
+      <c r="A115" s="60" t="n">
+        <v>87</v>
+      </c>
+      <c r="B115" s="60" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C115" s="60" t="inlineStr"/>
+      <c r="D115" s="60" t="inlineStr"/>
+      <c r="E115" s="60" t="inlineStr"/>
+      <c r="F115" s="58" t="n"/>
+      <c r="G115" s="58" t="n"/>
+      <c r="H115" s="60" t="inlineStr"/>
+      <c r="I115" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J115" s="60" t="inlineStr"/>
+    </row>
+    <row r="116" ht="16" customHeight="1" s="28">
+      <c r="A116" s="57" t="n">
+        <v>88</v>
+      </c>
+      <c r="B116" s="57" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="C116" s="57" t="inlineStr"/>
+      <c r="D116" s="57" t="inlineStr"/>
+      <c r="E116" s="57" t="inlineStr"/>
+      <c r="F116" s="58" t="n"/>
+      <c r="G116" s="58" t="n"/>
+      <c r="H116" s="57" t="inlineStr"/>
+      <c r="I116" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J116" s="57" t="inlineStr"/>
+    </row>
+    <row r="117"/>
+    <row r="118" ht="18" customHeight="1" s="28">
+      <c r="A118" s="145" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="16" customHeight="1" s="28">
+      <c r="A119" s="60" t="n">
+        <v>89</v>
+      </c>
+      <c r="B119" s="60" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="C119" s="60" t="inlineStr"/>
+      <c r="D119" s="60" t="inlineStr"/>
+      <c r="E119" s="60" t="inlineStr"/>
+      <c r="F119" s="58" t="n"/>
+      <c r="G119" s="58" t="n"/>
+      <c r="H119" s="60" t="inlineStr"/>
+      <c r="I119" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J119" s="60" t="inlineStr"/>
+    </row>
+    <row r="120" ht="16" customHeight="1" s="28">
+      <c r="A120" s="57" t="n">
+        <v>90</v>
+      </c>
+      <c r="B120" s="57" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="C120" s="57" t="inlineStr"/>
+      <c r="D120" s="57" t="inlineStr"/>
+      <c r="E120" s="57" t="inlineStr"/>
+      <c r="F120" s="58" t="n"/>
+      <c r="G120" s="58" t="n"/>
+      <c r="H120" s="57" t="inlineStr"/>
+      <c r="I120" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J120" s="57" t="inlineStr"/>
+    </row>
+    <row r="121" ht="16" customHeight="1" s="28">
+      <c r="A121" s="60" t="n">
+        <v>91</v>
+      </c>
+      <c r="B121" s="60" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="C121" s="60" t="inlineStr"/>
+      <c r="D121" s="60" t="inlineStr"/>
+      <c r="E121" s="60" t="inlineStr"/>
+      <c r="F121" s="58" t="n"/>
+      <c r="G121" s="58" t="n"/>
+      <c r="H121" s="60" t="inlineStr"/>
+      <c r="I121" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J121" s="60" t="inlineStr"/>
+    </row>
+    <row r="122" ht="16" customHeight="1" s="28">
+      <c r="A122" s="57" t="n">
+        <v>92</v>
+      </c>
+      <c r="B122" s="57" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="C122" s="57" t="inlineStr"/>
+      <c r="D122" s="57" t="inlineStr"/>
+      <c r="E122" s="57" t="inlineStr"/>
+      <c r="F122" s="58" t="n"/>
+      <c r="G122" s="58" t="n"/>
+      <c r="H122" s="57" t="inlineStr"/>
+      <c r="I122" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J122" s="57" t="inlineStr"/>
+    </row>
+    <row r="123" ht="16" customHeight="1" s="28">
+      <c r="A123" s="60" t="n">
+        <v>93</v>
+      </c>
+      <c r="B123" s="60" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="C123" s="60" t="inlineStr"/>
+      <c r="D123" s="60" t="inlineStr"/>
+      <c r="E123" s="60" t="inlineStr"/>
+      <c r="F123" s="58" t="n"/>
+      <c r="G123" s="58" t="n"/>
+      <c r="H123" s="60" t="inlineStr"/>
+      <c r="I123" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J123" s="60" t="inlineStr"/>
+    </row>
+    <row r="124" ht="16" customHeight="1" s="28">
+      <c r="A124" s="57" t="n">
+        <v>94</v>
+      </c>
+      <c r="B124" s="57" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="C124" s="57" t="inlineStr"/>
+      <c r="D124" s="57" t="inlineStr"/>
+      <c r="E124" s="57" t="inlineStr"/>
+      <c r="F124" s="58" t="n"/>
+      <c r="G124" s="58" t="n"/>
+      <c r="H124" s="57" t="inlineStr"/>
+      <c r="I124" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J124" s="57" t="inlineStr"/>
+    </row>
+    <row r="125" ht="16" customHeight="1" s="28">
+      <c r="A125" s="60" t="n">
+        <v>95</v>
+      </c>
+      <c r="B125" s="60" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="C125" s="60" t="inlineStr"/>
+      <c r="D125" s="60" t="inlineStr"/>
+      <c r="E125" s="60" t="inlineStr"/>
+      <c r="F125" s="58" t="n"/>
+      <c r="G125" s="58" t="n"/>
+      <c r="H125" s="60" t="inlineStr"/>
+      <c r="I125" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J125" s="60" t="inlineStr"/>
+    </row>
+    <row r="126" ht="16" customHeight="1" s="28">
+      <c r="A126" s="57" t="n">
+        <v>96</v>
+      </c>
+      <c r="B126" s="57" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="C126" s="57" t="inlineStr"/>
+      <c r="D126" s="57" t="inlineStr"/>
+      <c r="E126" s="57" t="inlineStr"/>
+      <c r="F126" s="58" t="n"/>
+      <c r="G126" s="58" t="n"/>
+      <c r="H126" s="57" t="inlineStr"/>
+      <c r="I126" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J126" s="57" t="inlineStr"/>
+    </row>
+    <row r="127"/>
+    <row r="128" ht="18" customHeight="1" s="28">
+      <c r="A128" s="145" t="inlineStr">
+        <is>
+          <t>Quarter-final</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="16" customHeight="1" s="28">
+      <c r="A129" s="60" t="n">
+        <v>97</v>
+      </c>
+      <c r="B129" s="60" t="inlineStr">
+        <is>
+          <t>Quarter-final</t>
+        </is>
+      </c>
+      <c r="C129" s="60" t="inlineStr"/>
+      <c r="D129" s="60" t="inlineStr"/>
+      <c r="E129" s="60" t="inlineStr"/>
+      <c r="F129" s="58" t="n"/>
+      <c r="G129" s="58" t="n"/>
+      <c r="H129" s="60" t="inlineStr"/>
+      <c r="I129" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J129" s="60" t="inlineStr"/>
+    </row>
+    <row r="130" ht="16" customHeight="1" s="28">
+      <c r="A130" s="57" t="n">
+        <v>98</v>
+      </c>
+      <c r="B130" s="57" t="inlineStr">
+        <is>
+          <t>Quarter-final</t>
+        </is>
+      </c>
+      <c r="C130" s="57" t="inlineStr"/>
+      <c r="D130" s="57" t="inlineStr"/>
+      <c r="E130" s="57" t="inlineStr"/>
+      <c r="F130" s="58" t="n"/>
+      <c r="G130" s="58" t="n"/>
+      <c r="H130" s="57" t="inlineStr"/>
+      <c r="I130" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J130" s="57" t="inlineStr"/>
+    </row>
+    <row r="131" ht="16" customHeight="1" s="28">
+      <c r="A131" s="60" t="n">
+        <v>99</v>
+      </c>
+      <c r="B131" s="60" t="inlineStr">
+        <is>
+          <t>Quarter-final</t>
+        </is>
+      </c>
+      <c r="C131" s="60" t="inlineStr"/>
+      <c r="D131" s="60" t="inlineStr"/>
+      <c r="E131" s="60" t="inlineStr"/>
+      <c r="F131" s="58" t="n"/>
+      <c r="G131" s="58" t="n"/>
+      <c r="H131" s="60" t="inlineStr"/>
+      <c r="I131" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J131" s="60" t="inlineStr"/>
+    </row>
+    <row r="132" ht="16" customHeight="1" s="28">
+      <c r="A132" s="57" t="n">
+        <v>100</v>
+      </c>
+      <c r="B132" s="57" t="inlineStr">
+        <is>
+          <t>Quarter-final</t>
+        </is>
+      </c>
+      <c r="C132" s="57" t="inlineStr"/>
+      <c r="D132" s="57" t="inlineStr"/>
+      <c r="E132" s="57" t="inlineStr"/>
+      <c r="F132" s="58" t="n"/>
+      <c r="G132" s="58" t="n"/>
+      <c r="H132" s="57" t="inlineStr"/>
+      <c r="I132" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J132" s="57" t="inlineStr"/>
+    </row>
+    <row r="133"/>
+    <row r="134" ht="18" customHeight="1" s="28">
+      <c r="A134" s="145" t="inlineStr">
+        <is>
+          <t>Semi-final</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="16" customHeight="1" s="28">
+      <c r="A135" s="60" t="n">
+        <v>101</v>
+      </c>
+      <c r="B135" s="60" t="inlineStr">
+        <is>
+          <t>Semi-final</t>
+        </is>
+      </c>
+      <c r="C135" s="60" t="inlineStr"/>
+      <c r="D135" s="60" t="inlineStr"/>
+      <c r="E135" s="60" t="inlineStr"/>
+      <c r="F135" s="58" t="n"/>
+      <c r="G135" s="58" t="n"/>
+      <c r="H135" s="60" t="inlineStr"/>
+      <c r="I135" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J135" s="60" t="inlineStr"/>
+    </row>
+    <row r="136" ht="16" customHeight="1" s="28">
+      <c r="A136" s="57" t="n">
+        <v>102</v>
+      </c>
+      <c r="B136" s="57" t="inlineStr">
+        <is>
+          <t>Semi-final</t>
+        </is>
+      </c>
+      <c r="C136" s="57" t="inlineStr"/>
+      <c r="D136" s="57" t="inlineStr"/>
+      <c r="E136" s="57" t="inlineStr"/>
+      <c r="F136" s="58" t="n"/>
+      <c r="G136" s="58" t="n"/>
+      <c r="H136" s="57" t="inlineStr"/>
+      <c r="I136" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J136" s="57" t="inlineStr"/>
+    </row>
+    <row r="137"/>
+    <row r="138" ht="18" customHeight="1" s="28">
+      <c r="A138" s="145" t="inlineStr">
+        <is>
+          <t>Third Place</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="16" customHeight="1" s="28">
+      <c r="A139" s="60" t="n">
+        <v>103</v>
+      </c>
+      <c r="B139" s="60" t="inlineStr">
+        <is>
+          <t>Third Place</t>
+        </is>
+      </c>
+      <c r="C139" s="60" t="inlineStr"/>
+      <c r="D139" s="60" t="inlineStr"/>
+      <c r="E139" s="60" t="inlineStr"/>
+      <c r="F139" s="58" t="n"/>
+      <c r="G139" s="58" t="n"/>
+      <c r="H139" s="60" t="inlineStr"/>
+      <c r="I139" s="60" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J139" s="60" t="inlineStr"/>
+    </row>
+    <row r="140"/>
+    <row r="141" ht="18" customHeight="1" s="28">
+      <c r="A141" s="145" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="16" customHeight="1" s="28">
+      <c r="A142" s="57" t="n">
+        <v>104</v>
+      </c>
+      <c r="B142" s="57" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C142" s="57" t="inlineStr"/>
+      <c r="D142" s="57" t="inlineStr"/>
+      <c r="E142" s="57" t="inlineStr"/>
+      <c r="F142" s="58" t="n"/>
+      <c r="G142" s="58" t="n"/>
+      <c r="H142" s="57" t="inlineStr"/>
+      <c r="I142" s="57" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="J142" s="57" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="A141:J141"/>
+    <mergeCell ref="A100:J100"/>
+    <mergeCell ref="A91:J91"/>
+    <mergeCell ref="A35:J35"/>
+    <mergeCell ref="A43:J43"/>
+    <mergeCell ref="A134:J134"/>
+    <mergeCell ref="A19:J19"/>
+    <mergeCell ref="A67:J67"/>
+    <mergeCell ref="A83:J83"/>
+    <mergeCell ref="A59:J59"/>
+    <mergeCell ref="A51:J51"/>
+    <mergeCell ref="A138:J138"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A128:J128"/>
+    <mergeCell ref="A99:J99"/>
+    <mergeCell ref="A118:J118"/>
+    <mergeCell ref="A75:J75"/>
+    <mergeCell ref="A27:J27"/>
+    <mergeCell ref="A3:J3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Show all tied badge winners in Statistics tab
- Twins badge now collects all pairs tied at the top Jaccard score,
  not just the first one
- write_badges_section renders one row per winner when there's a tie,
  with a 🏆 (tied) prefix, so every tied winner is clearly visible
  rather than being squeezed into a single cell

https://claude.ai/code/session_01VFqgqUhDsMbhjQyNveqHky
</commit_message>
<xml_diff>
--- a/WC2026_Pool.xlsx
+++ b/WC2026_Pool.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="49">
+  <fonts count="51">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -288,6 +288,18 @@
     <font>
       <i val="1"/>
       <color rgb="001C4587"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="007F2B00"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="001C4587"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="42">
@@ -636,7 +648,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -985,6 +997,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="41" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="40" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="41" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4595,7 +4613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="28" min="1" max="1"/>
@@ -6581,7 +6599,7 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="22" customHeight="1" s="28">
+    <row r="86" ht="20" customHeight="1" s="28">
       <c r="A86" s="104" t="inlineStr">
         <is>
           <t>⭐  Crowd Favourite</t>
@@ -6603,7 +6621,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="22" customHeight="1" s="28">
+    <row r="87" ht="20" customHeight="1" s="28">
       <c r="A87" s="107" t="inlineStr">
         <is>
           <t>🎯  Dark Horse</t>
@@ -6625,7 +6643,7 @@
         </is>
       </c>
     </row>
-    <row r="88" ht="22" customHeight="1" s="28">
+    <row r="88" ht="20" customHeight="1" s="28">
       <c r="A88" s="110" t="inlineStr">
         <is>
           <t>🐺  Lone Wolf</t>
@@ -6647,7 +6665,7 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="22" customHeight="1" s="28">
+    <row r="89" ht="20" customHeight="1" s="28">
       <c r="A89" s="113" t="inlineStr">
         <is>
           <t>🌍  Globetrotter</t>
@@ -6669,7 +6687,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="22" customHeight="1" s="28">
+    <row r="90" ht="20" customHeight="1" s="28">
       <c r="A90" s="116" t="inlineStr">
         <is>
           <t>🎲  Group Gambler</t>
@@ -6680,9 +6698,9 @@
           <t>Most picks from the same WC group — highest concentration risk</t>
         </is>
       </c>
-      <c r="D90" s="116" t="inlineStr">
-        <is>
-          <t>Ken Larade  /  Peter Miles</t>
+      <c r="D90" s="122" t="inlineStr">
+        <is>
+          <t>🏆 (tied)  Ken Larade</t>
         </is>
       </c>
       <c r="F90" s="118" t="inlineStr">
@@ -6691,30 +6709,50 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="22" customHeight="1" s="28">
-      <c r="A91" s="119" t="inlineStr">
+    <row r="91" ht="20" customHeight="1" s="28">
+      <c r="A91" s="116" t="inlineStr"/>
+      <c r="B91" s="117" t="inlineStr"/>
+      <c r="D91" s="122" t="inlineStr">
+        <is>
+          <t>🏆 (tied)  Peter Miles</t>
+        </is>
+      </c>
+      <c r="F91" s="118" t="inlineStr"/>
+    </row>
+    <row r="92" ht="20" customHeight="1" s="28">
+      <c r="A92" s="119" t="inlineStr">
         <is>
           <t>🤝  Twins</t>
         </is>
       </c>
-      <c r="B91" s="120" t="inlineStr">
+      <c r="B92" s="120" t="inlineStr">
         <is>
           <t>The pair of participants with the most picks in common</t>
         </is>
       </c>
-      <c r="D91" s="119" t="inlineStr">
-        <is>
-          <t>Ken Larade &amp; Lucie Kendell</t>
-        </is>
-      </c>
-      <c r="F91" s="121" t="inlineStr">
+      <c r="D92" s="123" t="inlineStr">
+        <is>
+          <t>🏆 (tied)  Ken Larade &amp; Lucie Kendell</t>
+        </is>
+      </c>
+      <c r="F92" s="121" t="inlineStr">
         <is>
           <t>5 shared picks (26% similarity): Belgium, Canada, Norway, Panama, Spain</t>
         </is>
       </c>
     </row>
+    <row r="93" ht="20" customHeight="1" s="28">
+      <c r="A93" s="119" t="inlineStr"/>
+      <c r="B93" s="120" t="inlineStr"/>
+      <c r="D93" s="123" t="inlineStr">
+        <is>
+          <t>🏆 (tied)  Lucie Kendell &amp; Peter Miles</t>
+        </is>
+      </c>
+      <c r="F93" s="121" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="37">
+  <mergeCells count="41">
     <mergeCell ref="B91:C91"/>
     <mergeCell ref="A84:F84"/>
     <mergeCell ref="B90:C90"/>
@@ -6722,6 +6760,7 @@
     <mergeCell ref="A80:F80"/>
     <mergeCell ref="D90:E90"/>
     <mergeCell ref="A74:F74"/>
+    <mergeCell ref="B93:C93"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="B71:F71"/>
     <mergeCell ref="A3:F3"/>
@@ -6739,6 +6778,7 @@
     <mergeCell ref="D87:E87"/>
     <mergeCell ref="A68:F68"/>
     <mergeCell ref="A58:F58"/>
+    <mergeCell ref="D93:E93"/>
     <mergeCell ref="A83:F83"/>
     <mergeCell ref="A48:F48"/>
     <mergeCell ref="A30:F30"/>
@@ -6746,6 +6786,8 @@
     <mergeCell ref="A59:F59"/>
     <mergeCell ref="A82:C82"/>
     <mergeCell ref="D81:F81"/>
+    <mergeCell ref="B92:C92"/>
+    <mergeCell ref="D92:E92"/>
     <mergeCell ref="A60:F60"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B89:C89"/>

</xml_diff>

<commit_message>
Add continental badges and fix reverted Twins badge
New badges:
- Around the World (🌐): picks span the most confederations/continents
- Continental Loyalist (🗺️): most picks concentrated in one confederation

Both use a CONFEDERATION map covering all 48 WC 2026 teams across
5 regions (Europe, South America, N. & C. America, Africa, Asia & Oceania).

Also restores the Twins badge tie-handling (show all pairs tied at the
top Jaccard score) which was lost in a prior rebase.

https://claude.ai/code/session_01VFqgqUhDsMbhjQyNveqHky
</commit_message>
<xml_diff>
--- a/WC2026_Pool.xlsx
+++ b/WC2026_Pool.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="49">
+  <fonts count="53">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -289,8 +289,24 @@
       <i val="1"/>
       <color rgb="001C4587"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000B3D6E"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="000B3D6E"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00660000"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00660000"/>
+    </font>
   </fonts>
-  <fills count="42">
+  <fills count="44">
     <fill>
       <patternFill/>
     </fill>
@@ -497,6 +513,16 @@
         <fgColor rgb="00CFE2F3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D0E4F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="12">
     <border>
@@ -636,7 +662,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -985,6 +1011,24 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="41" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="42" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="42" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="42" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="43" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="43" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="43" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4595,7 +4639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="28" min="1" max="1"/>
@@ -6692,29 +6736,73 @@
       </c>
     </row>
     <row r="91" ht="22" customHeight="1" s="28">
-      <c r="A91" s="119" t="inlineStr">
+      <c r="A91" s="122" t="inlineStr">
+        <is>
+          <t>🌐  Around the World</t>
+        </is>
+      </c>
+      <c r="B91" s="123" t="inlineStr">
+        <is>
+          <t>Picks span the most confederations/continents</t>
+        </is>
+      </c>
+      <c r="D91" s="122" t="inlineStr">
+        <is>
+          <t>Ryan Lowe  /  Lucie Kendell  /  Peter Miles</t>
+        </is>
+      </c>
+      <c r="F91" s="124" t="inlineStr">
+        <is>
+          <t>4 confederation(s) represented</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="22" customHeight="1" s="28">
+      <c r="A92" s="125" t="inlineStr">
+        <is>
+          <t>🗺️  Continental Loyalist</t>
+        </is>
+      </c>
+      <c r="B92" s="126" t="inlineStr">
+        <is>
+          <t>Most picks concentrated in a single confederation/continent</t>
+        </is>
+      </c>
+      <c r="D92" s="125" t="inlineStr">
+        <is>
+          <t>Ken Larade</t>
+        </is>
+      </c>
+      <c r="F92" s="127" t="inlineStr">
+        <is>
+          <t>7 picks from Europe: Belgium, Croatia, France, Norway, Scotland, Spain, Turkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1" s="28">
+      <c r="A93" s="119" t="inlineStr">
         <is>
           <t>🤝  Twins</t>
         </is>
       </c>
-      <c r="B91" s="120" t="inlineStr">
+      <c r="B93" s="120" t="inlineStr">
         <is>
           <t>The pair of participants with the most picks in common</t>
         </is>
       </c>
-      <c r="D91" s="119" t="inlineStr">
-        <is>
-          <t>Ken Larade &amp; Lucie Kendell</t>
-        </is>
-      </c>
-      <c r="F91" s="121" t="inlineStr">
+      <c r="D93" s="119" t="inlineStr">
+        <is>
+          <t>Ken Larade &amp; Lucie Kendell  /  Lucie Kendell &amp; Peter Miles</t>
+        </is>
+      </c>
+      <c r="F93" s="121" t="inlineStr">
         <is>
           <t>5 shared picks (26% similarity): Belgium, Canada, Norway, Panama, Spain</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="37">
+  <mergeCells count="41">
     <mergeCell ref="B91:C91"/>
     <mergeCell ref="A84:F84"/>
     <mergeCell ref="B90:C90"/>
@@ -6722,6 +6810,7 @@
     <mergeCell ref="A80:F80"/>
     <mergeCell ref="D90:E90"/>
     <mergeCell ref="A74:F74"/>
+    <mergeCell ref="B93:C93"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="B71:F71"/>
     <mergeCell ref="A3:F3"/>
@@ -6739,6 +6828,7 @@
     <mergeCell ref="D87:E87"/>
     <mergeCell ref="A68:F68"/>
     <mergeCell ref="A58:F58"/>
+    <mergeCell ref="D93:E93"/>
     <mergeCell ref="A83:F83"/>
     <mergeCell ref="A48:F48"/>
     <mergeCell ref="A30:F30"/>
@@ -6746,6 +6836,8 @@
     <mergeCell ref="A59:F59"/>
     <mergeCell ref="A82:C82"/>
     <mergeCell ref="D81:F81"/>
+    <mergeCell ref="B92:C92"/>
+    <mergeCell ref="D92:E92"/>
     <mergeCell ref="A60:F60"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B89:C89"/>

</xml_diff>